<commit_message>
Batch 1 builds: laptop grader, Axol workspace map, MARS odometry check, MorphoAI page
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K6KjNKe9qCXHsofcBCunE2
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="351" uniqueCount="272">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="271">
   <si>
     <t xml:space="preserve">#</t>
   </si>
@@ -141,649 +141,646 @@
     <t xml:space="preserve">Polymath Robotics</t>
   </si>
   <si>
+    <t xml:space="preserve">Ilia Baranov</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ilia@polymathrobotics.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">guess</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Autonomy software for industrial vehicles (tractors, mining trucks) controlled through a REST API. Free simulator called Caladan.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">API reference pages for /v2/relative-waypoints and /v2/polymath-feedback show no request or response fields (VERIFY in a browser: synapse.docs.polymathrobotics.dev/docs/api/relative-waypoints). Homepage tab title shows "Autonomy &amp;amp; Safety". Planned Caladan build was blocked: the API needs credentials from Polymath support.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Two small things in the Synapse API docs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Caladan is free and uses a REST API instead of ROS. Best build target in this batch.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">companies/01-02-polymath-robotics.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.polymathrobotics.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.ycombinator.com/companies/polymath-robotics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Innate</t>
+  </si>
+  <si>
     <t xml:space="preserve">A</t>
   </si>
   <si>
-    <t xml:space="preserve">Ilia Baranov</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ilia@polymathrobotics.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">guess</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Autonomy software for industrial vehicles (tractors, mining trucks) controlled through a REST API. Free simulator called Caladan.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BUILD: a Python behavior for the free Caladan sim (farm environment). Bonus: homepage browser tab shows "Autonomy &amp;amp; Safety" instead of "&amp;".</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Caladan Python behavior (farm env), e.g. waypoint row coverage with a simple PID heading controller</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Built a small behavior in Caladan</t>
+    <t xml:space="preserve">Vignesh Anand</t>
+  </si>
+  <si>
+    <t xml:space="preserve">vignesh@innate.bot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Personal AI robot (MARS, $995) you teach with code, language, and demonstrations. Open-source Innate OS plus a browser simulator.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BUILD (done): odometry-drift check skill for Innate OS. Bonus: site says "Teach MARS a task with one example" in one section and "Teach with a few examples" in another.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DONE: builds/innate-odom-check (odometry vs lidar drift check skill, tested on a fake robot, not on MARS/sim yet)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wrote an odometry-drift check skill for MARS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Careers page says degrees don't matter. Strong fit.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">companies/01-03-innate.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://innate.bot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.ycombinator.com/companies/innate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Almond</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Saba Khalilnaji</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Co-founder &amp; CEO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">saba@almond.bot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">guess (public: hello@almond.bot)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Axol, a dual-arm robot for physical AI ($9,499) with an open-source Python SDK, IK, and VR teleop.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BUILD (done): two-arm workspace map from the Axol URDF. Bonus: FAQ says two arms give "double the cycle time" of one arm, which reads like the opposite of what's meant (half the cycle time).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DONE: builds/almond-axol-workspace (bimanual reachability map from the SDK's URDF)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mapped Axol's two-arm workspace from your URDF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hiring Founding Robotics SWE. Ships from SF.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">companies/01-04-almond.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://almond.bot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.ycombinator.com/companies/almond</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MorphoAI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Andrew Spielberg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">andrew@morpho.ai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">guess (public: hello@morpho.ai)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI tool that generates, checks, and refines manufacturable designs for robots and machines. Backed by a 2.5M GBP ARIA grant.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BUILD (done): morpho.ai currently shows only the company name, no product description. Draft a one-page landing page from their YC launch description.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DONE: builds/morphoai-homepage-draft (one-page HTML, labeled unofficial)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Drafted a homepage for morpho.ai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hiring is London-based. Site is a near-empty Squarespace page.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">companies/01-05-morphoai.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://morpho.ai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.ycombinator.com/companies/morphoai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OS3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rishabh Chanana</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Founder</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rishabh@os3robotics.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Low-cost semi-humanoid robots (HALE 1.0). Developer units $14,995. First deployments in hotels.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Developer units are $14,995 but the site lists no payload, reach, runtime, weight, or compute. Offer to draft a spec table. Also meta description says "hospitality laundry" while the page just says "Hospitality".</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spec sheet idea for HALE developer units</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2-person team, very early. Contract mechanical role open.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">companies/01-06-os3.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://os3robotics.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.ycombinator.com/companies/os3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Darwin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sergio Charles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Founder &amp; CEO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sergio@darwinrobotics.ai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">General-purpose robots that learn by demonstration to assemble and maintain AI infrastructure. First deployments planned early 2027.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The "See it work" button points to #work but there doesn't seem to be a section with that id (VERIFY: click it).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"See it work" button on darwinrobotics.ai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weak value item. Verify the button before sending, or skip.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">companies/01-07-darwin.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://darwinrobotics.ai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.ycombinator.com/companies/darwin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lightberry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stephan Koenigstorfer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stephan@lightberry.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI "social brain" for robots so they can listen, speak, and act. Runs on Unitree, Booster, Fourier humanoids. Robot named Lumi.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Idea: use sound direction-of-arrival so the robot turns toward whoever is speaking. Venkat's HRTF engine is the reverse of that problem. Site note: homepage has one line about Lumi and no specs or details.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUDIO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spatial audio guy, interested in robots that listen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hiring Voice AI SWE. Good match for the audio project.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">companies/01-08-lightberry.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://lightberry.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.ycombinator.com/companies/lightberry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bucket Robotics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Matt Puchalski</t>
+  </si>
+  <si>
+    <t xml:space="preserve">matt@bucket.bot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Defect detection for manufacturing: CAD files in, vision model out, runs on edge devices like Jetson Orin Nano.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Homepage sets a large-image social card but has no preview image, so links shared on X/Slack/LinkedIn show up blank (VERIFY with a link preview checker like opengraph.xyz).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Link previews for bucket.bot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hiring ML, full stack, forward deploy.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">companies/01-09-bucket-robotics.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://bucket.bot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.ycombinator.com/companies/bucket-robotics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Saphira AI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Akshay Chalana</t>
+  </si>
+  <si>
+    <t xml:space="preserve">akshay@saphira.ai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">guess (public: contact@saphira.ai)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI agents that help hardware and robot companies get safety certified (ISO 10218, ISO 26262, UL, CE).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Customer quote from RobCo has no named speaker or title, which weakens it (VERIFY).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Robotics student curious about safety certification</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weaker fit. Lower priority.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">companies/01-10-saphira-ai.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://saphira.ai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.ycombinator.com/companies/saphira-ai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yondu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Michael Chen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">michael@yondu.ai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">guess (public: hello@yonduai.com)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Warehouse robots for order picking at 3PLs: teleop first (ULTRON), then autonomy (YGM). Has a Fall 2026 Mechatronics Intern posting.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Site is yondu.ai but the contact email is hello@yonduai.com (different domain). Copy also switches between "bin-picking" and "warehouse tasks" as the first thing you fully automate.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mechatronics intern question (and a small site note)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Has an intern posting. Michael helped build an open-source bipedal robot at MIT.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">companies/01-11-yondu.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://yondu.ai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.ycombinator.com/companies/yondu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ultra</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oliver Ortlieb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">oliver@ultra.tech</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OP1 stationary robots that pack and sort orders in warehouses. Raised $62M on Oct 9, 2026 and partnered with Physical Intelligence.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The "Introducing" section shows leftover CMS text: "No frames yet. Paste a manifest URL..." (VERIFY).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Placeholder text showing on ultra.tech</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fresh $62M raise, 19 open roles. Bigger hiring process, lower odds of cold reply but worth one shot.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">companies/01-12-ultra.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://ultra.tech</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.ycombinator.com/companies/ultra</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Proception</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jay Li</t>
+  </si>
+  <si>
+    <t xml:space="preserve">jay@proception.ai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dexterous robot hands (ProHand, 22 DOF, tactile skin) and a data glove (ProGlove). $11M seed led by First Round.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Explore products" button points to #products but there's no products section on the homepage. Nav says "Product", footer says "Products". (VERIFY)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Explore products" button on proception.ai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Only role open is a technician in Palo Alto.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">companies/01-13-proception.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://proception.ai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.ycombinator.com/companies/proception</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mbodi AI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sebastian Peralta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sebastian@mbodi.ai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Teach industrial robots new skills with plain language and demos. ABB partnership. Open-source embodied-agents library.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Every item in the press carousel links to the same TechInAsia article, including the TechCrunch and ABB headlines (VERIFY by clicking 3-4).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Press links on mbodi.ai all go to one article</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Could upgrade to a build later with their open-source embodied-agents library.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">companies/01-14-mbodi-ai.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.mbodi.ai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.ycombinator.com/companies/mbodi-ai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Orangewood Labs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Abhinav Das</t>
+  </si>
+  <si>
+    <t xml:space="preserve">abhinav@orangewood.co</t>
+  </si>
+  <si>
+    <t xml:space="preserve">guess (public: hellorobot@orangewood.co)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Affordable AI robot arms for small manufacturers (RoboGPT). Most of the team is in India.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The "Tasks Done by Orangewood Robots" section has the "rough estimates" disclaimer but no actual numbers showing (VERIFY).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Missing numbers in "Tasks Done by Orangewood Robots"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open roles are all in Noida. Lower priority.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">companies/01-15-orangewood-labs.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.orangewood.co</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.ycombinator.com/companies/orangewood-labs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Revise Robotics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rupesh Jeyaram</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rupesh@reviserobotics.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Robots that test, wipe, photograph, and list used laptops for resale. Posting Engineering Intern (Summer/Fall 2026).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BUILD (done): a Python script that pulls a laptop's battery wear, disk health, RAM, and CPU into a one-page resale grade report.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DONE: builds/revise-laptop-grader (Windows/macOS/Linux, tested grading rules)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Built a laptop health-check script for refurbishing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Has an Engineering Intern posting. Site didn't render for research; verify it loads.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">companies/01-16-revise-robotics.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.reviserobotics.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.ycombinator.com/companies/revise-robotics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aktoria Robotics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shreenabh Agrawal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">founders@aktoria.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">public (founders@ shown on site)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24/7 remote robot operators plus low-latency teleop software. Also sells teleop training data.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Site names "R1 Teleop" as a product but never explains it, and "works with any robot" has no list of supported platforms.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Question about R1 Teleop</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brand new (S26), 2 people. Public founders@ email.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">companies/01-17-aktoria-robotics.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://aktoria.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.ycombinator.com/companies/aktoria-robotics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Starcloud</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adi Oltean</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Founder &amp; Chief Engineer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">adi@starcloud.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data centers in space. Launched Starcloud-1 with an Nvidia H100 in Nov 2025. $170M Series A in Mar 2026.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOCAL: Venkat is in Redmond, same as Starcloud's hiring location, so he can help in person. Site footer still says (c) 2024 (VERIFY).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Redmond student who'd love to help in person</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Local in Redmond. Big company now ($1.1B), so lower cold-email odds, but the local angle is strong.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">companies/01-18-starcloud.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.starcloud.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.ycombinator.com/companies/starcloud</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Feather</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aahan Sawhney</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Co-founder</t>
+  </si>
+  <si>
+    <t xml:space="preserve">aahan@featherhq.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Voice AI platform for natural-sounding AI phone calls.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Site description used in Google results and link previews reads "Feather is helps enterprises build and deploy AI agents" (VERIFY by searching featherhq).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Typo in Feather's Google/link preview text</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Only open role is India-based. Lower priority.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">companies/01-19-feather.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.featherhq.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.ycombinator.com/companies/feather</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Silurian</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nikhil Shankar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Co-founder &amp; Chief Engineer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nikhil@silurian.ai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Foundation models that simulate Earth, starting with weather (GFT, 1.5B params). API for energy, insurance, agriculture.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Footer "API" link goes to the weather product page, not API docs (VERIFY).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">STOCK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Footer "API" link on silurian.ai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ML research role is senior. Lower priority.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">companies/01-20-silurian.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://silurian.ai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.ycombinator.com/companies/silurian</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metric</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Count</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Companies</t>
   </si>
   <si>
     <t xml:space="preserve">Waiting on build</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Caladan is free and uses a REST API instead of ROS. Best build target in this batch.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">companies/01-02-polymath-robotics.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.polymathrobotics.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.ycombinator.com/companies/polymath-robotics</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Innate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vignesh Anand</t>
-  </si>
-  <si>
-    <t xml:space="preserve">vignesh@innate.bot</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Personal AI robot (MARS, $995) you teach with code, language, and demonstrations. Open-source Innate OS plus a browser simulator.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BUILD: a skill in Innate OS run in sim.innate.bot. Bonus: site says "Teach MARS a task with one example" in one section and "Teach with a few examples" in another.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Innate OS skill in sim.innate.bot (github.com/innate-inc/innate-os)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Made a MARS skill in your simulator</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Careers page says degrees don't matter. Strong fit.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">companies/01-03-innate.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://innate.bot</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.ycombinator.com/companies/innate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Almond</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Saba Khalilnaji</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Co-founder &amp; CEO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">saba@almond.bot</t>
-  </si>
-  <si>
-    <t xml:space="preserve">guess (public: hello@almond.bot)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Axol, a dual-arm robot for physical AI ($9,499) with an open-source Python SDK, IK, and VR teleop.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BUILD: small tool/example on the open-source Axol SDK (github.com/almond-bot/axol). Bonus: FAQ says two arms give "double the cycle time" of one arm, which reads like the opposite of what's meant (half the cycle time).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Example/tool on the Axol Python SDK (no hardware needed), e.g. IK reachability visualizer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Something small I built with the Axol SDK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hiring Founding Robotics SWE. Ships from SF.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">companies/01-04-almond.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://almond.bot</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.ycombinator.com/companies/almond</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MorphoAI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Andrew Spielberg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">andrew@morpho.ai</t>
-  </si>
-  <si>
-    <t xml:space="preserve">guess (public: hello@morpho.ai)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AI tool that generates, checks, and refines manufacturable designs for robots and machines. Backed by a 2.5M GBP ARIA grant.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BUILD: morpho.ai currently shows only the company name, no product description. Draft a one-page landing page from their YC launch description.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Single-page landing page draft (HTML) from public YC launch copy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Drafted a homepage for morpho.ai</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hiring is London-based. Site is a near-empty Squarespace page.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">companies/01-05-morphoai.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://morpho.ai</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.ycombinator.com/companies/morphoai</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OS3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rishabh Chanana</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Founder</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rishabh@os3robotics.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Low-cost semi-humanoid robots (HALE 1.0). Developer units $14,995. First deployments in hotels.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Developer units are $14,995 but the site lists no payload, reach, runtime, weight, or compute. Offer to draft a spec table. Also meta description says "hospitality laundry" while the page just says "Hospitality".</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Spec sheet idea for HALE developer units</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2-person team, very early. Contract mechanical role open.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">companies/01-06-os3.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://os3robotics.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.ycombinator.com/companies/os3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Darwin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sergio Charles</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Founder &amp; CEO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sergio@darwinrobotics.ai</t>
-  </si>
-  <si>
-    <t xml:space="preserve">General-purpose robots that learn by demonstration to assemble and maintain AI infrastructure. First deployments planned early 2027.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The "See it work" button points to #work but there doesn't seem to be a section with that id (VERIFY: click it).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">"See it work" button on darwinrobotics.ai</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Weak value item. Verify the button before sending, or skip.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">companies/01-07-darwin.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://darwinrobotics.ai</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.ycombinator.com/companies/darwin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lightberry</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stephan Koenigstorfer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">stephan@lightberry.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AI "social brain" for robots so they can listen, speak, and act. Runs on Unitree, Booster, Fourier humanoids. Robot named Lumi.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Idea: use sound direction-of-arrival so the robot turns toward whoever is speaking. Venkat's HRTF engine is the reverse of that problem. Site note: homepage has one line about Lumi and no specs or details.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUDIO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Spatial audio guy, interested in robots that listen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hiring Voice AI SWE. Good match for the audio project.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">companies/01-08-lightberry.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://lightberry.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.ycombinator.com/companies/lightberry</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bucket Robotics</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Matt Puchalski</t>
-  </si>
-  <si>
-    <t xml:space="preserve">matt@bucket.bot</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Defect detection for manufacturing: CAD files in, vision model out, runs on edge devices like Jetson Orin Nano.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Homepage sets a large-image social card but has no preview image, so links shared on X/Slack/LinkedIn show up blank (VERIFY with a link preview checker like opengraph.xyz).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Link previews for bucket.bot</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hiring ML, full stack, forward deploy.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">companies/01-09-bucket-robotics.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://bucket.bot</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.ycombinator.com/companies/bucket-robotics</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Saphira AI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Akshay Chalana</t>
-  </si>
-  <si>
-    <t xml:space="preserve">akshay@saphira.ai</t>
-  </si>
-  <si>
-    <t xml:space="preserve">guess (public: contact@saphira.ai)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AI agents that help hardware and robot companies get safety certified (ISO 10218, ISO 26262, UL, CE).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Customer quote from RobCo has no named speaker or title, which weakens it (VERIFY).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Robotics student curious about safety certification</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Weaker fit. Lower priority.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">companies/01-10-saphira-ai.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://saphira.ai</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.ycombinator.com/companies/saphira-ai</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yondu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Michael Chen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">michael@yondu.ai</t>
-  </si>
-  <si>
-    <t xml:space="preserve">guess (public: hello@yonduai.com)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Warehouse robots for order picking at 3PLs: teleop first (ULTRON), then autonomy (YGM). Has a Fall 2026 Mechatronics Intern posting.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Site is yondu.ai but the contact email is hello@yonduai.com (different domain). Copy also switches between "bin-picking" and "warehouse tasks" as the first thing you fully automate.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mechatronics intern question (and a small site note)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Has an intern posting. Michael helped build an open-source bipedal robot at MIT.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">companies/01-11-yondu.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://yondu.ai</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.ycombinator.com/companies/yondu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ultra</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Oliver Ortlieb</t>
-  </si>
-  <si>
-    <t xml:space="preserve">oliver@ultra.tech</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OP1 stationary robots that pack and sort orders in warehouses. Raised $62M on Oct 9, 2026 and partnered with Physical Intelligence.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The "Introducing" section shows leftover CMS text: "No frames yet. Paste a manifest URL..." (VERIFY).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Placeholder text showing on ultra.tech</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fresh $62M raise, 19 open roles. Bigger hiring process, lower odds of cold reply but worth one shot.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">companies/01-12-ultra.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://ultra.tech</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.ycombinator.com/companies/ultra</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Proception</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jay Li</t>
-  </si>
-  <si>
-    <t xml:space="preserve">jay@proception.ai</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dexterous robot hands (ProHand, 22 DOF, tactile skin) and a data glove (ProGlove). $11M seed led by First Round.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">"Explore products" button points to #products but there's no products section on the homepage. Nav says "Product", footer says "Products". (VERIFY)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">"Explore products" button on proception.ai</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Only role open is a technician in Palo Alto.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">companies/01-13-proception.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://proception.ai</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.ycombinator.com/companies/proception</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mbodi AI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sebastian Peralta</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sebastian@mbodi.ai</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Teach industrial robots new skills with plain language and demos. ABB partnership. Open-source embodied-agents library.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Every item in the press carousel links to the same TechInAsia article, including the TechCrunch and ABB headlines (VERIFY by clicking 3-4).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Press links on mbodi.ai all go to one article</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Could upgrade to a build later with their open-source embodied-agents library.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">companies/01-14-mbodi-ai.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.mbodi.ai</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.ycombinator.com/companies/mbodi-ai</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Orangewood Labs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Abhinav Das</t>
-  </si>
-  <si>
-    <t xml:space="preserve">abhinav@orangewood.co</t>
-  </si>
-  <si>
-    <t xml:space="preserve">guess (public: hellorobot@orangewood.co)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Affordable AI robot arms for small manufacturers (RoboGPT). Most of the team is in India.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The "Tasks Done by Orangewood Robots" section has the "rough estimates" disclaimer but no actual numbers showing (VERIFY).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Missing numbers in "Tasks Done by Orangewood Robots"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Open roles are all in Noida. Lower priority.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">companies/01-15-orangewood-labs.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.orangewood.co</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.ycombinator.com/companies/orangewood-labs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Revise Robotics</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rupesh Jeyaram</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rupesh@reviserobotics.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Robots that test, wipe, photograph, and list used laptops for resale. Posting Engineering Intern (Summer/Fall 2026).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BUILD: a Python script that pulls a laptop's battery wear, disk health, RAM, and CPU into a one-page resale grade report.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Python laptop health report (battery wear, SMART disk status, RAM, CPU) with a resale grade</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Built a laptop health-check script for refurbishing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Has an Engineering Intern posting. Site didn't render for research; verify it loads.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">companies/01-16-revise-robotics.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.reviserobotics.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.ycombinator.com/companies/revise-robotics</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aktoria Robotics</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Shreenabh Agrawal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">founders@aktoria.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">public (founders@ shown on site)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">24/7 remote robot operators plus low-latency teleop software. Also sells teleop training data.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Site names "R1 Teleop" as a product but never explains it, and "works with any robot" has no list of supported platforms.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Question about R1 Teleop</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Brand new (S26), 2 people. Public founders@ email.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">companies/01-17-aktoria-robotics.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://aktoria.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.ycombinator.com/companies/aktoria-robotics</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Starcloud</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Adi Oltean</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Founder &amp; Chief Engineer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">adi@starcloud.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Data centers in space. Launched Starcloud-1 with an Nvidia H100 in Nov 2025. $170M Series A in Mar 2026.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LOCAL: Venkat is in Redmond, same as Starcloud's hiring location, so he can help in person. Site footer still says (c) 2024 (VERIFY).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Redmond student who'd love to help in person</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Local in Redmond. Big company now ($1.1B), so lower cold-email odds, but the local angle is strong.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">companies/01-18-starcloud.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.starcloud.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.ycombinator.com/companies/starcloud</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Feather</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aahan Sawhney</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Co-founder</t>
-  </si>
-  <si>
-    <t xml:space="preserve">aahan@featherhq.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Voice AI platform for natural-sounding AI phone calls.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Site description used in Google results and link previews reads "Feather is helps enterprises build and deploy AI agents" (VERIFY by searching featherhq).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Typo in Feather's Google/link preview text</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Only open role is India-based. Lower priority.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">companies/01-19-feather.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.featherhq.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.ycombinator.com/companies/feather</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Silurian</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nikhil Shankar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Co-founder &amp; Chief Engineer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nikhil@silurian.ai</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Foundation models that simulate Earth, starting with weather (GFT, 1.5B params). API for energy, insurance, agriculture.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Footer "API" link goes to the weather product page, not API docs (VERIFY).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">STOCK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Footer "API" link on silurian.ai</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ML research role is senior. Lower priority.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">companies/01-20-silurian.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://silurian.ai</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.ycombinator.com/companies/silurian</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Metric</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Count</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Companies</t>
   </si>
   <si>
     <t xml:space="preserve">Verified</t>
@@ -1453,7 +1450,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="n">
         <v>2</v>
       </c>
@@ -1464,37 +1461,35 @@
         <v>37</v>
       </c>
       <c r="D3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>38</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>39</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>25</v>
       </c>
       <c r="G3" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="H3" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="I3" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="J3" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="J3" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="K3" s="2" t="s">
-        <v>44</v>
-      </c>
+      <c r="K3" s="2"/>
       <c r="L3" s="2" t="s">
         <v>30</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="N3" s="3" t="s">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="O3" s="4"/>
       <c r="P3" s="5" t="str">
@@ -1504,19 +1499,19 @@
       <c r="Q3" s="4"/>
       <c r="R3" s="3"/>
       <c r="S3" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="T3" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="U3" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="V3" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="T3" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="U3" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="V3" s="6" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="4" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
@@ -1524,40 +1519,40 @@
         <v>1</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>38</v>
+        <v>49</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>25</v>
       </c>
       <c r="G4" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="J4" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="H4" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="I4" s="2" t="s">
+      <c r="K4" s="2" t="s">
         <v>54</v>
-      </c>
-      <c r="J4" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="K4" s="2" t="s">
-        <v>56</v>
       </c>
       <c r="L4" s="2" t="s">
         <v>30</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="N4" s="3" t="s">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="O4" s="4"/>
       <c r="P4" s="5" t="str">
@@ -1567,19 +1562,19 @@
       <c r="Q4" s="4"/>
       <c r="R4" s="3"/>
       <c r="S4" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="T4" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="U4" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="T4" s="2" t="s">
+      <c r="V4" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="U4" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="V4" s="6" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="5" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="n">
         <v>4</v>
       </c>
@@ -1587,40 +1582,40 @@
         <v>1</v>
       </c>
       <c r="C5" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="F5" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="D5" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="E5" s="2" t="s">
+      <c r="G5" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="H5" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="I5" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="H5" s="2" t="s">
+      <c r="J5" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="I5" s="2" t="s">
+      <c r="K5" s="2" t="s">
         <v>67</v>
-      </c>
-      <c r="J5" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="K5" s="2" t="s">
-        <v>69</v>
       </c>
       <c r="L5" s="2" t="s">
         <v>30</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="N5" s="3" t="s">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="O5" s="4"/>
       <c r="P5" s="5" t="str">
@@ -1630,16 +1625,16 @@
       <c r="Q5" s="4"/>
       <c r="R5" s="3"/>
       <c r="S5" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="T5" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="U5" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="T5" s="2" t="s">
+      <c r="V5" s="6" t="s">
         <v>72</v>
-      </c>
-      <c r="U5" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="V5" s="6" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1650,40 +1645,40 @@
         <v>1</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>38</v>
+        <v>49</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>25</v>
       </c>
       <c r="G6" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="I6" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="H6" s="2" t="s">
+      <c r="J6" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="I6" s="2" t="s">
+      <c r="K6" s="2" t="s">
         <v>79</v>
-      </c>
-      <c r="J6" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="K6" s="2" t="s">
-        <v>81</v>
       </c>
       <c r="L6" s="2" t="s">
         <v>30</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="N6" s="3" t="s">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="O6" s="4"/>
       <c r="P6" s="5" t="str">
@@ -1693,16 +1688,16 @@
       <c r="Q6" s="4"/>
       <c r="R6" s="3"/>
       <c r="S6" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="T6" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="U6" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="T6" s="2" t="s">
+      <c r="V6" s="6" t="s">
         <v>84</v>
-      </c>
-      <c r="U6" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="V6" s="6" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1713,35 +1708,35 @@
         <v>1</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>23</v>
       </c>
       <c r="E7" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="G7" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="H7" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="I7" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="J7" s="2" t="s">
         <v>90</v>
-      </c>
-      <c r="H7" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="I7" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="J7" s="2" t="s">
-        <v>92</v>
       </c>
       <c r="K7" s="2"/>
       <c r="L7" s="2" t="s">
         <v>30</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="N7" s="3" t="s">
         <v>32</v>
@@ -1754,16 +1749,16 @@
       <c r="Q7" s="4"/>
       <c r="R7" s="3"/>
       <c r="S7" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="T7" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="U7" s="6" t="s">
         <v>94</v>
       </c>
-      <c r="T7" s="2" t="s">
+      <c r="V7" s="6" t="s">
         <v>95</v>
-      </c>
-      <c r="U7" s="6" t="s">
-        <v>96</v>
-      </c>
-      <c r="V7" s="6" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1774,35 +1769,35 @@
         <v>1</v>
       </c>
       <c r="C8" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="E8" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="F8" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="G8" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="H8" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="I8" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="G8" s="2" t="s">
+      <c r="J8" s="2" t="s">
         <v>102</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="I8" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="J8" s="2" t="s">
-        <v>104</v>
       </c>
       <c r="K8" s="2"/>
       <c r="L8" s="2" t="s">
         <v>30</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="N8" s="3" t="s">
         <v>32</v>
@@ -1815,16 +1810,16 @@
       <c r="Q8" s="4"/>
       <c r="R8" s="3"/>
       <c r="S8" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="T8" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="U8" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="T8" s="2" t="s">
+      <c r="V8" s="6" t="s">
         <v>107</v>
-      </c>
-      <c r="U8" s="6" t="s">
-        <v>108</v>
-      </c>
-      <c r="V8" s="6" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1835,35 +1830,35 @@
         <v>1</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>23</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>25</v>
       </c>
       <c r="G9" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="J9" s="2" t="s">
         <v>112</v>
-      </c>
-      <c r="H9" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="I9" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="J9" s="2" t="s">
-        <v>114</v>
       </c>
       <c r="K9" s="2"/>
       <c r="L9" s="2" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="N9" s="3" t="s">
         <v>32</v>
@@ -1876,16 +1871,16 @@
       <c r="Q9" s="4"/>
       <c r="R9" s="3"/>
       <c r="S9" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="T9" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="U9" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="T9" s="2" t="s">
+      <c r="V9" s="6" t="s">
         <v>118</v>
-      </c>
-      <c r="U9" s="6" t="s">
-        <v>119</v>
-      </c>
-      <c r="V9" s="6" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1896,35 +1891,35 @@
         <v>1</v>
       </c>
       <c r="C10" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="G10" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="D10" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="E10" s="2" t="s">
+      <c r="H10" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="I10" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="F10" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="G10" s="2" t="s">
+      <c r="J10" s="2" t="s">
         <v>123</v>
-      </c>
-      <c r="H10" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="I10" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="J10" s="2" t="s">
-        <v>125</v>
       </c>
       <c r="K10" s="2"/>
       <c r="L10" s="2" t="s">
         <v>30</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="N10" s="3" t="s">
         <v>32</v>
@@ -1937,16 +1932,16 @@
       <c r="Q10" s="4"/>
       <c r="R10" s="3"/>
       <c r="S10" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="T10" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="U10" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="T10" s="2" t="s">
+      <c r="V10" s="6" t="s">
         <v>128</v>
-      </c>
-      <c r="U10" s="6" t="s">
-        <v>129</v>
-      </c>
-      <c r="V10" s="6" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1957,35 +1952,35 @@
         <v>1</v>
       </c>
       <c r="C11" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="G11" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="D11" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="E11" s="2" t="s">
+      <c r="H11" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="F11" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="G11" s="2" t="s">
+      <c r="I11" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="H11" s="2" t="s">
+      <c r="J11" s="2" t="s">
         <v>134</v>
-      </c>
-      <c r="I11" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="J11" s="2" t="s">
-        <v>136</v>
       </c>
       <c r="K11" s="2"/>
       <c r="L11" s="2" t="s">
         <v>30</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="N11" s="3" t="s">
         <v>32</v>
@@ -1998,16 +1993,16 @@
       <c r="Q11" s="4"/>
       <c r="R11" s="3"/>
       <c r="S11" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="T11" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="U11" s="6" t="s">
         <v>138</v>
       </c>
-      <c r="T11" s="2" t="s">
+      <c r="V11" s="6" t="s">
         <v>139</v>
-      </c>
-      <c r="U11" s="6" t="s">
-        <v>140</v>
-      </c>
-      <c r="V11" s="6" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2018,35 +2013,35 @@
         <v>1</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>23</v>
       </c>
       <c r="E12" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="H12" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="F12" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="G12" s="2" t="s">
+      <c r="I12" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="H12" s="2" t="s">
+      <c r="J12" s="2" t="s">
         <v>145</v>
-      </c>
-      <c r="I12" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="J12" s="2" t="s">
-        <v>147</v>
       </c>
       <c r="K12" s="2"/>
       <c r="L12" s="2" t="s">
         <v>30</v>
       </c>
       <c r="M12" s="2" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="N12" s="3" t="s">
         <v>32</v>
@@ -2059,16 +2054,16 @@
       <c r="Q12" s="4"/>
       <c r="R12" s="3"/>
       <c r="S12" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="T12" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="U12" s="6" t="s">
         <v>149</v>
       </c>
-      <c r="T12" s="2" t="s">
+      <c r="V12" s="6" t="s">
         <v>150</v>
-      </c>
-      <c r="U12" s="6" t="s">
-        <v>151</v>
-      </c>
-      <c r="V12" s="6" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2079,35 +2074,35 @@
         <v>1</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>23</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>25</v>
       </c>
       <c r="G13" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="J13" s="2" t="s">
         <v>155</v>
-      </c>
-      <c r="H13" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="I13" s="2" t="s">
-        <v>156</v>
-      </c>
-      <c r="J13" s="2" t="s">
-        <v>157</v>
       </c>
       <c r="K13" s="2"/>
       <c r="L13" s="2" t="s">
         <v>30</v>
       </c>
       <c r="M13" s="2" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="N13" s="3" t="s">
         <v>32</v>
@@ -2120,16 +2115,16 @@
       <c r="Q13" s="4"/>
       <c r="R13" s="3"/>
       <c r="S13" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="T13" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="U13" s="6" t="s">
         <v>159</v>
       </c>
-      <c r="T13" s="2" t="s">
+      <c r="V13" s="6" t="s">
         <v>160</v>
-      </c>
-      <c r="U13" s="6" t="s">
-        <v>161</v>
-      </c>
-      <c r="V13" s="6" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2140,35 +2135,35 @@
         <v>1</v>
       </c>
       <c r="C14" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="G14" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="D14" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="E14" s="2" t="s">
+      <c r="H14" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="I14" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="F14" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="G14" s="2" t="s">
+      <c r="J14" s="2" t="s">
         <v>165</v>
-      </c>
-      <c r="H14" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="I14" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="J14" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="K14" s="2"/>
       <c r="L14" s="2" t="s">
         <v>30</v>
       </c>
       <c r="M14" s="2" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="N14" s="3" t="s">
         <v>32</v>
@@ -2181,16 +2176,16 @@
       <c r="Q14" s="4"/>
       <c r="R14" s="3"/>
       <c r="S14" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="T14" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="U14" s="6" t="s">
         <v>169</v>
       </c>
-      <c r="T14" s="2" t="s">
+      <c r="V14" s="6" t="s">
         <v>170</v>
-      </c>
-      <c r="U14" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="V14" s="6" t="s">
-        <v>172</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2201,35 +2196,35 @@
         <v>1</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>23</v>
       </c>
       <c r="E15" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="I15" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="F15" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="G15" s="2" t="s">
+      <c r="J15" s="2" t="s">
         <v>175</v>
-      </c>
-      <c r="H15" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="I15" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="J15" s="2" t="s">
-        <v>177</v>
       </c>
       <c r="K15" s="2"/>
       <c r="L15" s="2" t="s">
         <v>30</v>
       </c>
       <c r="M15" s="2" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="N15" s="3" t="s">
         <v>32</v>
@@ -2242,16 +2237,16 @@
       <c r="Q15" s="4"/>
       <c r="R15" s="3"/>
       <c r="S15" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="T15" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="U15" s="6" t="s">
         <v>179</v>
       </c>
-      <c r="T15" s="2" t="s">
+      <c r="V15" s="6" t="s">
         <v>180</v>
-      </c>
-      <c r="U15" s="6" t="s">
-        <v>181</v>
-      </c>
-      <c r="V15" s="6" t="s">
-        <v>182</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2262,35 +2257,35 @@
         <v>1</v>
       </c>
       <c r="C16" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="G16" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="D16" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="E16" s="2" t="s">
+      <c r="H16" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="F16" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="G16" s="2" t="s">
+      <c r="I16" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="H16" s="2" t="s">
+      <c r="J16" s="2" t="s">
         <v>186</v>
-      </c>
-      <c r="I16" s="2" t="s">
-        <v>187</v>
-      </c>
-      <c r="J16" s="2" t="s">
-        <v>188</v>
       </c>
       <c r="K16" s="2"/>
       <c r="L16" s="2" t="s">
         <v>30</v>
       </c>
       <c r="M16" s="2" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="N16" s="3" t="s">
         <v>32</v>
@@ -2303,16 +2298,16 @@
       <c r="Q16" s="4"/>
       <c r="R16" s="3"/>
       <c r="S16" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="T16" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="U16" s="6" t="s">
         <v>190</v>
       </c>
-      <c r="T16" s="2" t="s">
+      <c r="V16" s="6" t="s">
         <v>191</v>
-      </c>
-      <c r="U16" s="6" t="s">
-        <v>192</v>
-      </c>
-      <c r="V16" s="6" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2323,40 +2318,40 @@
         <v>1</v>
       </c>
       <c r="C17" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="G17" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="D17" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="E17" s="2" t="s">
+      <c r="H17" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="I17" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="F17" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="G17" s="2" t="s">
+      <c r="J17" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="H17" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="I17" s="2" t="s">
+      <c r="K17" s="2" t="s">
         <v>197</v>
-      </c>
-      <c r="J17" s="2" t="s">
-        <v>198</v>
-      </c>
-      <c r="K17" s="2" t="s">
-        <v>199</v>
       </c>
       <c r="L17" s="2" t="s">
         <v>30</v>
       </c>
       <c r="M17" s="2" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="N17" s="3" t="s">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="O17" s="4"/>
       <c r="P17" s="5" t="str">
@@ -2366,16 +2361,16 @@
       <c r="Q17" s="4"/>
       <c r="R17" s="3"/>
       <c r="S17" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="T17" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="U17" s="6" t="s">
         <v>201</v>
       </c>
-      <c r="T17" s="2" t="s">
+      <c r="V17" s="6" t="s">
         <v>202</v>
-      </c>
-      <c r="U17" s="6" t="s">
-        <v>203</v>
-      </c>
-      <c r="V17" s="6" t="s">
-        <v>204</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2386,35 +2381,35 @@
         <v>1</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>23</v>
       </c>
       <c r="E18" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="H18" s="2" t="s">
         <v>206</v>
       </c>
-      <c r="F18" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="G18" s="2" t="s">
+      <c r="I18" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="H18" s="2" t="s">
+      <c r="J18" s="2" t="s">
         <v>208</v>
-      </c>
-      <c r="I18" s="2" t="s">
-        <v>209</v>
-      </c>
-      <c r="J18" s="2" t="s">
-        <v>210</v>
       </c>
       <c r="K18" s="2"/>
       <c r="L18" s="2" t="s">
         <v>30</v>
       </c>
       <c r="M18" s="2" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="N18" s="3" t="s">
         <v>32</v>
@@ -2427,16 +2422,16 @@
       <c r="Q18" s="4"/>
       <c r="R18" s="3"/>
       <c r="S18" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="T18" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="U18" s="6" t="s">
         <v>212</v>
       </c>
-      <c r="T18" s="2" t="s">
+      <c r="V18" s="6" t="s">
         <v>213</v>
-      </c>
-      <c r="U18" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="V18" s="6" t="s">
-        <v>215</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2447,35 +2442,35 @@
         <v>1</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>23</v>
       </c>
       <c r="E19" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="G19" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="F19" s="2" t="s">
+      <c r="H19" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="I19" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="G19" s="2" t="s">
+      <c r="J19" s="2" t="s">
         <v>219</v>
-      </c>
-      <c r="H19" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="I19" s="2" t="s">
-        <v>220</v>
-      </c>
-      <c r="J19" s="2" t="s">
-        <v>221</v>
       </c>
       <c r="K19" s="2"/>
       <c r="L19" s="2" t="s">
         <v>30</v>
       </c>
       <c r="M19" s="2" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="N19" s="3" t="s">
         <v>32</v>
@@ -2488,16 +2483,16 @@
       <c r="Q19" s="4"/>
       <c r="R19" s="3"/>
       <c r="S19" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="T19" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="U19" s="6" t="s">
         <v>223</v>
       </c>
-      <c r="T19" s="2" t="s">
+      <c r="V19" s="6" t="s">
         <v>224</v>
-      </c>
-      <c r="U19" s="6" t="s">
-        <v>225</v>
-      </c>
-      <c r="V19" s="6" t="s">
-        <v>226</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2508,35 +2503,35 @@
         <v>1</v>
       </c>
       <c r="C20" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="F20" s="2" t="s">
         <v>227</v>
       </c>
-      <c r="D20" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="E20" s="2" t="s">
+      <c r="G20" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="F20" s="2" t="s">
+      <c r="H20" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="I20" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="G20" s="2" t="s">
+      <c r="J20" s="2" t="s">
         <v>230</v>
-      </c>
-      <c r="H20" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="I20" s="2" t="s">
-        <v>231</v>
-      </c>
-      <c r="J20" s="2" t="s">
-        <v>232</v>
       </c>
       <c r="K20" s="2"/>
       <c r="L20" s="2" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="M20" s="2" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="N20" s="3" t="s">
         <v>32</v>
@@ -2549,16 +2544,16 @@
       <c r="Q20" s="4"/>
       <c r="R20" s="3"/>
       <c r="S20" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="T20" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="U20" s="6" t="s">
         <v>234</v>
       </c>
-      <c r="T20" s="2" t="s">
+      <c r="V20" s="6" t="s">
         <v>235</v>
-      </c>
-      <c r="U20" s="6" t="s">
-        <v>236</v>
-      </c>
-      <c r="V20" s="6" t="s">
-        <v>237</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2569,35 +2564,35 @@
         <v>1</v>
       </c>
       <c r="C21" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="F21" s="2" t="s">
         <v>238</v>
       </c>
-      <c r="D21" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="E21" s="2" t="s">
+      <c r="G21" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="F21" s="2" t="s">
+      <c r="H21" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="I21" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="G21" s="2" t="s">
+      <c r="J21" s="2" t="s">
         <v>241</v>
-      </c>
-      <c r="H21" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="I21" s="2" t="s">
-        <v>242</v>
-      </c>
-      <c r="J21" s="2" t="s">
-        <v>243</v>
       </c>
       <c r="K21" s="2"/>
       <c r="L21" s="2" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="M21" s="2" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="N21" s="3" t="s">
         <v>32</v>
@@ -2610,16 +2605,16 @@
       <c r="Q21" s="4"/>
       <c r="R21" s="3"/>
       <c r="S21" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="T21" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="U21" s="6" t="s">
         <v>246</v>
       </c>
-      <c r="T21" s="2" t="s">
+      <c r="V21" s="6" t="s">
         <v>247</v>
-      </c>
-      <c r="U21" s="6" t="s">
-        <v>248</v>
-      </c>
-      <c r="V21" s="6" t="s">
-        <v>249</v>
       </c>
     </row>
   </sheetData>
@@ -2697,15 +2692,15 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="B2" s="8" t="n">
         <f aca="false">COUNTA(Tracker!C2:C21)</f>
@@ -2714,11 +2709,11 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>46</v>
+        <v>251</v>
       </c>
       <c r="B3" s="8" t="n">
         <f aca="false">COUNTIF(Tracker!N2:N21,"Waiting on build")</f>
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2727,12 +2722,12 @@
       </c>
       <c r="B4" s="8" t="n">
         <f aca="false">COUNTIF(Tracker!N2:N21,"Ready to review")</f>
-        <v>15</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B5" s="8" t="n">
         <f aca="false">COUNTIF(Tracker!N2:N21,"Verified")</f>
@@ -2741,7 +2736,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B6" s="8" t="n">
         <f aca="false">COUNTIF(Tracker!N2:N21,"Sent")</f>
@@ -2750,7 +2745,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B7" s="8" t="n">
         <f aca="false">COUNTIF(Tracker!N2:N21,"Followed up")</f>
@@ -2759,7 +2754,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B8" s="8" t="n">
         <f aca="false">COUNTIF(Tracker!N2:N21,"Replied")</f>
@@ -2768,7 +2763,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B9" s="8" t="n">
         <f aca="false">COUNTIF(Tracker!N2:N21,"Call scheduled")</f>
@@ -2777,7 +2772,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B10" s="8" t="n">
         <f aca="false">COUNTIF(Tracker!N2:N21,"No reply")</f>
@@ -2786,7 +2781,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B11" s="8" t="n">
         <f aca="false">COUNTIF(Tracker!N2:N21,"Skip")</f>
@@ -2799,25 +2794,25 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B13" s="8" t="n">
         <f aca="false">COUNTIF(Tracker!D2:D21,"A")</f>
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="8" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B14" s="8" t="n">
         <f aca="false">COUNTIF(Tracker!D2:D21,"B")</f>
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B15" s="8" t="n">
         <f aca="false">COUNTIF(Tracker!D2:D21,"C")</f>
@@ -2830,7 +2825,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B17" s="9" t="str">
         <f aca="false">IFERROR((B8+B9)/(B6+B7+B8+B9+B10),"-")</f>
@@ -2861,42 +2856,42 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Link each build to its own repo; turn 4 drafts into follow-ups on August threads
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K6KjNKe9qCXHsofcBCunE2
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="271">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="272">
   <si>
     <t xml:space="preserve">#</t>
   </si>
@@ -189,7 +189,7 @@
     <t xml:space="preserve">BUILD (done): odometry-drift check skill for Innate OS. Bonus: site says "Teach MARS a task with one example" in one section and "Teach with a few examples" in another.</t>
   </si>
   <si>
-    <t xml:space="preserve">DONE: builds/innate-odom-check (odometry vs lidar drift check skill, tested on a fake robot, not on MARS/sim yet)</t>
+    <t xml:space="preserve">DONE: github.com/Venkat960407/mars-odometry-check (odometry vs lidar drift check skill, tested on a fake robot, not on MARS/sim yet)</t>
   </si>
   <si>
     <t xml:space="preserve">Wrote an odometry-drift check skill for MARS</t>
@@ -228,7 +228,7 @@
     <t xml:space="preserve">BUILD (done): two-arm workspace map from the Axol URDF. Bonus: FAQ says two arms give "double the cycle time" of one arm, which reads like the opposite of what's meant (half the cycle time).</t>
   </si>
   <si>
-    <t xml:space="preserve">DONE: builds/almond-axol-workspace (bimanual reachability map from the SDK's URDF)</t>
+    <t xml:space="preserve">DONE: github.com/Venkat960407/axol-workspace-map (bimanual reachability map from the SDK's URDF)</t>
   </si>
   <si>
     <t xml:space="preserve">Mapped Axol's two-arm workspace from your URDF</t>
@@ -264,7 +264,7 @@
     <t xml:space="preserve">BUILD (done): morpho.ai currently shows only the company name, no product description. Draft a one-page landing page from their YC launch description.</t>
   </si>
   <si>
-    <t xml:space="preserve">DONE: builds/morphoai-homepage-draft (one-page HTML, labeled unofficial)</t>
+    <t xml:space="preserve">DONE: github.com/Venkat960407/morphoai-homepage-draft (one-page HTML, labeled unofficial)</t>
   </si>
   <si>
     <t xml:space="preserve">Drafted a homepage for morpho.ai</t>
@@ -291,7 +291,10 @@
     <t xml:space="preserve">Founder</t>
   </si>
   <si>
-    <t xml:space="preserve">rishabh@os3robotics.com</t>
+    <t xml:space="preserve">hi@os3robotics.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">emailed Aug 15, no bounce (draft is a reply in that thread)</t>
   </si>
   <si>
     <t xml:space="preserve">Low-cost semi-humanoid robots (HALE 1.0). Developer units $14,995. First deployments in hotels.</t>
@@ -357,7 +360,7 @@
     <t xml:space="preserve">Stephan Koenigstorfer</t>
   </si>
   <si>
-    <t xml:space="preserve">stephan@lightberry.com</t>
+    <t xml:space="preserve">founders@lightberry.com</t>
   </si>
   <si>
     <t xml:space="preserve">AI "social brain" for robots so they can listen, speak, and act. Runs on Unitree, Booster, Fourier humanoids. Robot named Lumi.</t>
@@ -486,7 +489,7 @@
     <t xml:space="preserve">Oliver Ortlieb</t>
   </si>
   <si>
-    <t xml:space="preserve">oliver@ultra.tech</t>
+    <t xml:space="preserve">founders@ultra.tech</t>
   </si>
   <si>
     <t xml:space="preserve">OP1 stationary robots that pack and sort orders in warehouses. Raised $62M on Oct 9, 2026 and partnered with Physical Intelligence.</t>
@@ -618,7 +621,7 @@
     <t xml:space="preserve">BUILD (done): a Python script that pulls a laptop's battery wear, disk health, RAM, and CPU into a one-page resale grade report.</t>
   </si>
   <si>
-    <t xml:space="preserve">DONE: builds/revise-laptop-grader (Windows/macOS/Linux, tested grading rules)</t>
+    <t xml:space="preserve">DONE: github.com/Venkat960407/laptop-resale-grader (Windows/macOS/Linux, tested grading rules)</t>
   </si>
   <si>
     <t xml:space="preserve">Built a laptop health-check script for refurbishing</t>
@@ -1511,7 +1514,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
@@ -1574,7 +1577,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="n">
         <v>4</v>
       </c>
@@ -1637,7 +1640,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="n">
         <v>5</v>
       </c>
@@ -1723,20 +1726,20 @@
         <v>88</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>40</v>
+        <v>89</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="K7" s="2"/>
       <c r="L7" s="2" t="s">
         <v>30</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="N7" s="3" t="s">
         <v>32</v>
@@ -1749,16 +1752,16 @@
       <c r="Q7" s="4"/>
       <c r="R7" s="3"/>
       <c r="S7" s="3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="T7" s="2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="U7" s="6" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="V7" s="6" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1769,35 +1772,35 @@
         <v>1</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="H8" s="2" t="s">
         <v>40</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="K8" s="2"/>
       <c r="L8" s="2" t="s">
         <v>30</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="N8" s="3" t="s">
         <v>32</v>
@@ -1810,16 +1813,16 @@
       <c r="Q8" s="4"/>
       <c r="R8" s="3"/>
       <c r="S8" s="3" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="T8" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="U8" s="6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="V8" s="6" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1830,35 +1833,35 @@
         <v>1</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>23</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>25</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>40</v>
+        <v>89</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="K9" s="2"/>
       <c r="L9" s="2" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="N9" s="3" t="s">
         <v>32</v>
@@ -1871,16 +1874,16 @@
       <c r="Q9" s="4"/>
       <c r="R9" s="3"/>
       <c r="S9" s="3" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="T9" s="2" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="U9" s="6" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="V9" s="6" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1891,35 +1894,35 @@
         <v>1</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H10" s="2" t="s">
         <v>40</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="K10" s="2"/>
       <c r="L10" s="2" t="s">
         <v>30</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="N10" s="3" t="s">
         <v>32</v>
@@ -1932,16 +1935,16 @@
       <c r="Q10" s="4"/>
       <c r="R10" s="3"/>
       <c r="S10" s="3" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="T10" s="2" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="U10" s="6" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="V10" s="6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1952,35 +1955,35 @@
         <v>1</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>62</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="K11" s="2"/>
       <c r="L11" s="2" t="s">
         <v>30</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="N11" s="3" t="s">
         <v>32</v>
@@ -1993,16 +1996,16 @@
       <c r="Q11" s="4"/>
       <c r="R11" s="3"/>
       <c r="S11" s="3" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="T11" s="2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="U11" s="6" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="V11" s="6" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2013,35 +2016,35 @@
         <v>1</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>23</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="K12" s="2"/>
       <c r="L12" s="2" t="s">
         <v>30</v>
       </c>
       <c r="M12" s="2" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="N12" s="3" t="s">
         <v>32</v>
@@ -2054,16 +2057,16 @@
       <c r="Q12" s="4"/>
       <c r="R12" s="3"/>
       <c r="S12" s="3" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="T12" s="2" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="U12" s="6" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="V12" s="6" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2074,35 +2077,35 @@
         <v>1</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>23</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>25</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>40</v>
+        <v>89</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="K13" s="2"/>
       <c r="L13" s="2" t="s">
         <v>30</v>
       </c>
       <c r="M13" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="N13" s="3" t="s">
         <v>32</v>
@@ -2115,16 +2118,16 @@
       <c r="Q13" s="4"/>
       <c r="R13" s="3"/>
       <c r="S13" s="3" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="T13" s="2" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="U13" s="6" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="V13" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2135,35 +2138,35 @@
         <v>1</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="H14" s="2" t="s">
         <v>40</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="K14" s="2"/>
       <c r="L14" s="2" t="s">
         <v>30</v>
       </c>
       <c r="M14" s="2" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="N14" s="3" t="s">
         <v>32</v>
@@ -2176,16 +2179,16 @@
       <c r="Q14" s="4"/>
       <c r="R14" s="3"/>
       <c r="S14" s="3" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="T14" s="2" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="U14" s="6" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="V14" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2196,35 +2199,35 @@
         <v>1</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>23</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="H15" s="2" t="s">
         <v>40</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K15" s="2"/>
       <c r="L15" s="2" t="s">
         <v>30</v>
       </c>
       <c r="M15" s="2" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="N15" s="3" t="s">
         <v>32</v>
@@ -2237,16 +2240,16 @@
       <c r="Q15" s="4"/>
       <c r="R15" s="3"/>
       <c r="S15" s="3" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="T15" s="2" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="U15" s="6" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="V15" s="6" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2257,35 +2260,35 @@
         <v>1</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="F16" s="2" t="s">
         <v>87</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="K16" s="2"/>
       <c r="L16" s="2" t="s">
         <v>30</v>
       </c>
       <c r="M16" s="2" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="N16" s="3" t="s">
         <v>32</v>
@@ -2298,19 +2301,19 @@
       <c r="Q16" s="4"/>
       <c r="R16" s="3"/>
       <c r="S16" s="3" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="T16" s="2" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="U16" s="6" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="V16" s="6" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="n">
         <v>16</v>
       </c>
@@ -2318,37 +2321,37 @@
         <v>1</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>49</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>40</v>
+        <v>89</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="L17" s="2" t="s">
         <v>30</v>
       </c>
       <c r="M17" s="2" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="N17" s="3" t="s">
         <v>32</v>
@@ -2361,16 +2364,16 @@
       <c r="Q17" s="4"/>
       <c r="R17" s="3"/>
       <c r="S17" s="3" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="T17" s="2" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="U17" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="V17" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2381,35 +2384,35 @@
         <v>1</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>23</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="F18" s="2" t="s">
         <v>87</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K18" s="2"/>
       <c r="L18" s="2" t="s">
         <v>30</v>
       </c>
       <c r="M18" s="2" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="N18" s="3" t="s">
         <v>32</v>
@@ -2422,16 +2425,16 @@
       <c r="Q18" s="4"/>
       <c r="R18" s="3"/>
       <c r="S18" s="3" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="T18" s="2" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="U18" s="6" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="V18" s="6" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2442,35 +2445,35 @@
         <v>1</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>23</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="H19" s="2" t="s">
         <v>40</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J19" s="2" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="K19" s="2"/>
       <c r="L19" s="2" t="s">
         <v>30</v>
       </c>
       <c r="M19" s="2" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="N19" s="3" t="s">
         <v>32</v>
@@ -2483,16 +2486,16 @@
       <c r="Q19" s="4"/>
       <c r="R19" s="3"/>
       <c r="S19" s="3" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="T19" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="U19" s="6" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="V19" s="6" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2503,35 +2506,35 @@
         <v>1</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="H20" s="2" t="s">
         <v>40</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="K20" s="2"/>
       <c r="L20" s="2" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="M20" s="2" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="N20" s="3" t="s">
         <v>32</v>
@@ -2544,16 +2547,16 @@
       <c r="Q20" s="4"/>
       <c r="R20" s="3"/>
       <c r="S20" s="3" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="T20" s="2" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="U20" s="6" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="V20" s="6" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2564,35 +2567,35 @@
         <v>1</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="H21" s="2" t="s">
         <v>40</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="J21" s="2" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="K21" s="2"/>
       <c r="L21" s="2" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="M21" s="2" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="N21" s="3" t="s">
         <v>32</v>
@@ -2605,16 +2608,16 @@
       <c r="Q21" s="4"/>
       <c r="R21" s="3"/>
       <c r="S21" s="3" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="T21" s="2" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="U21" s="6" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="V21" s="6" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
   </sheetData>
@@ -2692,15 +2695,15 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B2" s="8" t="n">
         <f aca="false">COUNTA(Tracker!C2:C21)</f>
@@ -2709,7 +2712,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B3" s="8" t="n">
         <f aca="false">COUNTIF(Tracker!N2:N21,"Waiting on build")</f>
@@ -2727,7 +2730,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B5" s="8" t="n">
         <f aca="false">COUNTIF(Tracker!N2:N21,"Verified")</f>
@@ -2736,7 +2739,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B6" s="8" t="n">
         <f aca="false">COUNTIF(Tracker!N2:N21,"Sent")</f>
@@ -2745,7 +2748,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B7" s="8" t="n">
         <f aca="false">COUNTIF(Tracker!N2:N21,"Followed up")</f>
@@ -2754,7 +2757,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="B8" s="8" t="n">
         <f aca="false">COUNTIF(Tracker!N2:N21,"Replied")</f>
@@ -2763,7 +2766,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B9" s="8" t="n">
         <f aca="false">COUNTIF(Tracker!N2:N21,"Call scheduled")</f>
@@ -2772,7 +2775,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B10" s="8" t="n">
         <f aca="false">COUNTIF(Tracker!N2:N21,"No reply")</f>
@@ -2781,7 +2784,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B11" s="8" t="n">
         <f aca="false">COUNTIF(Tracker!N2:N21,"Skip")</f>
@@ -2794,7 +2797,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B13" s="8" t="n">
         <f aca="false">COUNTIF(Tracker!D2:D21,"A")</f>
@@ -2803,7 +2806,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="8" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B14" s="8" t="n">
         <f aca="false">COUNTIF(Tracker!D2:D21,"B")</f>
@@ -2812,7 +2815,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B15" s="8" t="n">
         <f aca="false">COUNTIF(Tracker!D2:D21,"C")</f>
@@ -2825,7 +2828,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B17" s="9" t="str">
         <f aca="false">IFERROR((B8+B9)/(B6+B7+B8+B9+B10),"-")</f>
@@ -2856,42 +2859,42 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Use email-finder results in tracker; add Draft To/BCC columns; backup addresses on low-confidence drafts
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K6KjNKe9qCXHsofcBCunE2
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -13,7 +13,7 @@
     <sheet name="How to use" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Tracker!$A$1:$V$21</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Tracker!$A$1:$AC$21</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="272">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="465" uniqueCount="346">
   <si>
     <t xml:space="preserve">#</t>
   </si>
@@ -93,6 +93,27 @@
     <t xml:space="preserve">YC page</t>
   </si>
   <si>
+    <t xml:space="preserve">Draft To</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Draft BCC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Domain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Email confidence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Email source</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Email checked</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Email candidates</t>
+  </si>
+  <si>
     <t xml:space="preserve">Theseus</t>
   </si>
   <si>
@@ -138,6 +159,18 @@
     <t xml:space="preserve">https://www.ycombinator.com/companies/theseus</t>
   </si>
   <si>
+    <t xml:space="preserve">theseus.us</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pattern {first} from holden@theseus.us, ian@theseus.us</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-18 10:45</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sacha@theseus.us, sacha.levy@theseus.us, slevy@theseus.us, sachalevy@theseus.us, s.levy@theseus.us, sachal@theseus.us</t>
+  </si>
+  <si>
     <t xml:space="preserve">Polymath Robotics</t>
   </si>
   <si>
@@ -147,175 +180,229 @@
     <t xml:space="preserve">ilia@polymathrobotics.com</t>
   </si>
   <si>
+    <t xml:space="preserve">found</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Autonomy software for industrial vehicles (tractors, mining trucks) controlled through a REST API. Free simulator called Caladan.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">API reference pages for /v2/relative-waypoints and /v2/polymath-feedback show no request or response fields (VERIFY in a browser: synapse.docs.polymathrobotics.dev/docs/api/relative-waypoints). Homepage tab title shows "Autonomy &amp;amp; Safety". Planned Caladan build was blocked: the API needs credentials from Polymath support.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Two small things in the Synapse API docs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Caladan is free and uses a REST API instead of ROS. Best build target in this batch.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">companies/01-02-polymath-robotics.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.polymathrobotics.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.ycombinator.com/companies/polymath-robotics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">polymathrobotics.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://github.com/iliabaranov/rp2040-eth-keypad/commit/65c79007a22eb06245214527296f9995ad40dc4a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-18 01:17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ilia@polymathrobotics.com, ilia.baranov@polymathrobotics.com, ibaranov@polymathrobotics.com, iliabaranov@polymathrobotics.com, i.baranov@polymathrobotics.com, iliab@polymathrobotics.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Innate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vignesh Anand</t>
+  </si>
+  <si>
+    <t xml:space="preserve">vignesh@innate.bot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Personal AI robot (MARS, $995) you teach with code, language, and demonstrations. Open-source Innate OS plus a browser simulator.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BUILD (done): odometry-drift check skill for Innate OS. Bonus: site says "Teach MARS a task with one example" in one section and "Teach with a few examples" in another.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DONE: github.com/Venkat960407/mars-odometry-check (odometry vs lidar drift check skill, tested on a fake robot, not on MARS/sim yet)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wrote an odometry-drift check skill for MARS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Careers page says degrees don't matter. Strong fit.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">companies/01-03-innate.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://innate.bot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.ycombinator.com/companies/innate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">innate.bot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://github.com/innate-inc/GraspGen/commit/5ba3a4adf4484055523d4a82be431abefb185b01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">vignesh@innate.bot, vignesh.anand@innate.bot, vanand@innate.bot, vigneshanand@innate.bot, v.anand@innate.bot, vignesha@innate.bot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Almond</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Saba Khalilnaji</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Co-founder &amp; CEO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">saba@almond.bot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">guess (public: hello@almond.bot)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Axol, a dual-arm robot for physical AI ($9,499) with an open-source Python SDK, IK, and VR teleop.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BUILD (done): two-arm workspace map from the Axol URDF. Bonus: FAQ says two arms give "double the cycle time" of one arm, which reads like the opposite of what's meant (half the cycle time).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DONE: github.com/Venkat960407/axol-workspace-map (bimanual reachability map from the SDK's URDF)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mapped Axol's two-arm workspace from your URDF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hiring Founding Robotics SWE. Ships from SF.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">companies/01-04-almond.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://almond.bot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.ycombinator.com/companies/almond</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hello@almond.bot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">almond.bot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">prior {first} (11/11 indexed domains) (no personal addresses at this domain on site, DNS, YC, HN, Wayback, web or GitHub)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">saba@almond.bot, saba.khalilnaji@almond.bot, skhalilnaji@almond.bot, sabakhalilnaji@almond.bot, s.khalilnaji@almond.bot, sabak@almond.bot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MorphoAI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Andrew Spielberg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">andrew@morpho.ai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">guess (public: hello@morpho.ai)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI tool that generates, checks, and refines manufacturable designs for robots and machines. Backed by a 2.5M GBP ARIA grant.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BUILD (done): morpho.ai currently shows only the company name, no product description. Draft a one-page landing page from their YC launch description.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DONE: github.com/Venkat960407/morphoai-homepage-draft (one-page HTML, labeled unofficial)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Drafted a homepage for morpho.ai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hiring is London-based. Site is a near-empty Squarespace page.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">companies/01-05-morphoai.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://morpho.ai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.ycombinator.com/companies/morphoai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hello@morpho.ai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">morpho.ai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">prior {first} (11/11 indexed domains) (no personal addresses at this domain on site, DNS, YC, HN, Wayback, web or GitHub) | also seen on: morphoai.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">andrew@morpho.ai, andy@morpho.ai, andrew.spielberg@morpho.ai, aspielberg@morpho.ai, andrewspielberg@morpho.ai, a.spielberg@morpho.ai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OS3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rishabh Chanana</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Founder</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rishabh@os3robotics.com</t>
+  </si>
+  <si>
     <t xml:space="preserve">guess</t>
   </si>
   <si>
-    <t xml:space="preserve">Autonomy software for industrial vehicles (tractors, mining trucks) controlled through a REST API. Free simulator called Caladan.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">API reference pages for /v2/relative-waypoints and /v2/polymath-feedback show no request or response fields (VERIFY in a browser: synapse.docs.polymathrobotics.dev/docs/api/relative-waypoints). Homepage tab title shows "Autonomy &amp;amp; Safety". Planned Caladan build was blocked: the API needs credentials from Polymath support.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Two small things in the Synapse API docs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Caladan is free and uses a REST API instead of ROS. Best build target in this batch.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">companies/01-02-polymath-robotics.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.polymathrobotics.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.ycombinator.com/companies/polymath-robotics</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Innate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vignesh Anand</t>
-  </si>
-  <si>
-    <t xml:space="preserve">vignesh@innate.bot</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Personal AI robot (MARS, $995) you teach with code, language, and demonstrations. Open-source Innate OS plus a browser simulator.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BUILD (done): odometry-drift check skill for Innate OS. Bonus: site says "Teach MARS a task with one example" in one section and "Teach with a few examples" in another.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DONE: github.com/Venkat960407/mars-odometry-check (odometry vs lidar drift check skill, tested on a fake robot, not on MARS/sim yet)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wrote an odometry-drift check skill for MARS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Careers page says degrees don't matter. Strong fit.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">companies/01-03-innate.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://innate.bot</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.ycombinator.com/companies/innate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Almond</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Saba Khalilnaji</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Co-founder &amp; CEO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">saba@almond.bot</t>
-  </si>
-  <si>
-    <t xml:space="preserve">guess (public: hello@almond.bot)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Axol, a dual-arm robot for physical AI ($9,499) with an open-source Python SDK, IK, and VR teleop.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BUILD (done): two-arm workspace map from the Axol URDF. Bonus: FAQ says two arms give "double the cycle time" of one arm, which reads like the opposite of what's meant (half the cycle time).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DONE: github.com/Venkat960407/axol-workspace-map (bimanual reachability map from the SDK's URDF)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mapped Axol's two-arm workspace from your URDF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hiring Founding Robotics SWE. Ships from SF.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">companies/01-04-almond.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://almond.bot</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.ycombinator.com/companies/almond</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MorphoAI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Andrew Spielberg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">andrew@morpho.ai</t>
-  </si>
-  <si>
-    <t xml:space="preserve">guess (public: hello@morpho.ai)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AI tool that generates, checks, and refines manufacturable designs for robots and machines. Backed by a 2.5M GBP ARIA grant.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BUILD (done): morpho.ai currently shows only the company name, no product description. Draft a one-page landing page from their YC launch description.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DONE: github.com/Venkat960407/morphoai-homepage-draft (one-page HTML, labeled unofficial)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Drafted a homepage for morpho.ai</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hiring is London-based. Site is a near-empty Squarespace page.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">companies/01-05-morphoai.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://morpho.ai</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.ycombinator.com/companies/morphoai</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OS3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rishabh Chanana</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Founder</t>
+    <t xml:space="preserve">Low-cost semi-humanoid robots (HALE 1.0). Developer units $14,995. First deployments in hotels.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Developer units are $14,995 but the site lists no payload, reach, runtime, weight, or compute. Offer to draft a spec table. Also meta description says "hospitality laundry" while the page just says "Hospitality".</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spec sheet idea for HALE developer units</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2-person team, very early. Contract mechanical role open.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">companies/01-06-os3.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://os3robotics.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.ycombinator.com/companies/os3</t>
   </si>
   <si>
     <t xml:space="preserve">hi@os3robotics.com</t>
   </si>
   <si>
-    <t xml:space="preserve">emailed Aug 15, no bounce (draft is a reply in that thread)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Low-cost semi-humanoid robots (HALE 1.0). Developer units $14,995. First deployments in hotels.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Developer units are $14,995 but the site lists no payload, reach, runtime, weight, or compute. Offer to draft a spec table. Also meta description says "hospitality laundry" while the page just says "Hospitality".</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Spec sheet idea for HALE developer units</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2-person team, very early. Contract mechanical role open.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">companies/01-06-os3.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://os3robotics.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.ycombinator.com/companies/os3</t>
+    <t xml:space="preserve">os3robotics.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rishabh@os3robotics.com, rishabh.chanana@os3robotics.com, rchanana@os3robotics.com, rishabhchanana@os3robotics.com, r.chanana@os3robotics.com, rishabhc@os3robotics.com</t>
   </si>
   <si>
     <t xml:space="preserve">Darwin</t>
@@ -354,37 +441,61 @@
     <t xml:space="preserve">https://www.ycombinator.com/companies/darwin</t>
   </si>
   <si>
+    <t xml:space="preserve">ask@darwinrobotics.ai, sergio@thesislabs.ai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">darwinrobotics.ai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">prior {first} (11/11 indexed domains) (no personal addresses at this domain on site, DNS, YC, HN, Wayback, web or GitHub) | other real addresses: sergio@thesislabs.ai (published by the company), sergiogcharles@gmail.com (personal, GitHub sergiogcharles)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sergio@darwinrobotics.ai, sergio.charles@darwinrobotics.ai, scharles@darwinrobotics.ai, sergiocharles@darwinrobotics.ai, s.charles@darwinrobotics.ai, sergioc@darwinrobotics.ai</t>
+  </si>
+  <si>
     <t xml:space="preserve">Lightberry</t>
   </si>
   <si>
     <t xml:space="preserve">Stephan Koenigstorfer</t>
   </si>
   <si>
+    <t xml:space="preserve">stephan@lightberry.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI "social brain" for robots so they can listen, speak, and act. Runs on Unitree, Booster, Fourier humanoids. Robot named Lumi.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Idea: use sound direction-of-arrival so the robot turns toward whoever is speaking. Venkat's HRTF engine is the reverse of that problem. Site note: homepage has one line about Lumi and no specs or details.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUDIO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spatial audio guy, interested in robots that listen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hiring Voice AI SWE. Good match for the audio project.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">companies/01-08-lightberry.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://lightberry.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.ycombinator.com/companies/lightberry</t>
+  </si>
+  <si>
     <t xml:space="preserve">founders@lightberry.com</t>
   </si>
   <si>
-    <t xml:space="preserve">AI "social brain" for robots so they can listen, speak, and act. Runs on Unitree, Booster, Fourier humanoids. Robot named Lumi.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Idea: use sound direction-of-arrival so the robot turns toward whoever is speaking. Venkat's HRTF engine is the reverse of that problem. Site note: homepage has one line about Lumi and no specs or details.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUDIO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Spatial audio guy, interested in robots that listen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hiring Voice AI SWE. Good match for the audio project.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">companies/01-08-lightberry.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://lightberry.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.ycombinator.com/companies/lightberry</t>
+    <t xml:space="preserve">lightberry.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">prior {first} (11/11 indexed domains); ambiguous with Stephan Wolski (no personal addresses at this domain on site, DNS, YC, HN, Wayback, web or GitHub) | other real addresses: stephan.koenigstorfer@gmail.com (personal, GitHub sadkoeni)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stephan@lightberry.com, stephank@lightberry.com, stephan.koenigstorfer@lightberry.com, skoenigstorfer@lightberry.com, stephankoenigstorfer@lightberry.com, s.koenigstorfer@lightberry.com</t>
   </si>
   <si>
     <t xml:space="preserve">Bucket Robotics</t>
@@ -417,6 +528,18 @@
     <t xml:space="preserve">https://www.ycombinator.com/companies/bucket-robotics</t>
   </si>
   <si>
+    <t xml:space="preserve">bucket.bot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://news.ycombinator.com/item?id=41367750</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-18 01:42</t>
+  </si>
+  <si>
+    <t xml:space="preserve">matt@bucket.bot, matt.puchalski@bucket.bot, mpuchalski@bucket.bot, mattpuchalski@bucket.bot, m.puchalski@bucket.bot, mattp@bucket.bot</t>
+  </si>
+  <si>
     <t xml:space="preserve">Saphira AI</t>
   </si>
   <si>
@@ -426,9 +549,6 @@
     <t xml:space="preserve">akshay@saphira.ai</t>
   </si>
   <si>
-    <t xml:space="preserve">guess (public: contact@saphira.ai)</t>
-  </si>
-  <si>
     <t xml:space="preserve">AI agents that help hardware and robot companies get safety certified (ISO 10218, ISO 26262, UL, CE).</t>
   </si>
   <si>
@@ -450,13 +570,19 @@
     <t xml:space="preserve">https://www.ycombinator.com/companies/saphira-ai</t>
   </si>
   <si>
+    <t xml:space="preserve">saphira.ai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">akshay@saphira.ai, akshay.chalana@saphira.ai, achalana@saphira.ai, akshaychalana@saphira.ai, a.chalana@saphira.ai, akshayc@saphira.ai</t>
+  </si>
+  <si>
     <t xml:space="preserve">Yondu</t>
   </si>
   <si>
     <t xml:space="preserve">Michael Chen</t>
   </si>
   <si>
-    <t xml:space="preserve">michael@yondu.ai</t>
+    <t xml:space="preserve">michael@yonduai.com</t>
   </si>
   <si>
     <t xml:space="preserve">guess (public: hello@yonduai.com)</t>
@@ -483,34 +609,58 @@
     <t xml:space="preserve">https://www.ycombinator.com/companies/yondu</t>
   </si>
   <si>
+    <t xml:space="preserve">hello@yonduai.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">yondu.ai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">prior {first} (11/11 indexed domains) (no personal addresses at this domain on site, DNS, YC, HN, Wayback, web or GitHub) | mail domain yonduai.com, not yondu.ai (addresses only seen there)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">michael@yonduai.com, mike@yonduai.com, michael.chen@yonduai.com, mchen@yonduai.com, michaelchen@yonduai.com, m.chen@yonduai.com, michael@yondu.ai, mike@yondu.ai</t>
+  </si>
+  <si>
     <t xml:space="preserve">Ultra</t>
   </si>
   <si>
     <t xml:space="preserve">Oliver Ortlieb</t>
   </si>
   <si>
+    <t xml:space="preserve">oliver@ultra.tech</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OP1 stationary robots that pack and sort orders in warehouses. Raised $62M on Oct 9, 2026 and partnered with Physical Intelligence.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The "Introducing" section shows leftover CMS text: "No frames yet. Paste a manifest URL..." (VERIFY).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Placeholder text showing on ultra.tech</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fresh $62M raise, 19 open roles. Bigger hiring process, lower odds of cold reply but worth one shot.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">companies/01-12-ultra.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://ultra.tech</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.ycombinator.com/companies/ultra</t>
+  </si>
+  <si>
     <t xml:space="preserve">founders@ultra.tech</t>
   </si>
   <si>
-    <t xml:space="preserve">OP1 stationary robots that pack and sort orders in warehouses. Raised $62M on Oct 9, 2026 and partnered with Physical Intelligence.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The "Introducing" section shows leftover CMS text: "No frames yet. Paste a manifest URL..." (VERIFY).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Placeholder text showing on ultra.tech</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fresh $62M raise, 19 open roles. Bigger hiring process, lower odds of cold reply but worth one shot.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">companies/01-12-ultra.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://ultra.tech</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.ycombinator.com/companies/ultra</t>
+    <t xml:space="preserve">ultra.tech</t>
+  </si>
+  <si>
+    <t xml:space="preserve">prior {first} (11/11 indexed domains) (no personal addresses at this domain on site, DNS, YC, HN, Wayback, web or GitHub) | other real addresses: oortlieb@gmail.com (personal, GitHub oortlieb)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">oliver@ultra.tech, oliver.ortlieb@ultra.tech, oortlieb@ultra.tech, oliverortlieb@ultra.tech, o.ortlieb@ultra.tech, olivero@ultra.tech</t>
   </si>
   <si>
     <t xml:space="preserve">Proception</t>
@@ -543,6 +693,15 @@
     <t xml:space="preserve">https://www.ycombinator.com/companies/proception</t>
   </si>
   <si>
+    <t xml:space="preserve">proception.ai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://github.com/JayLiStanford/uniform-recycle/commit/ce458c5d632fc9f3c3ba206ebc4690bd07726f11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">jay@proception.ai, jay.li@proception.ai, jli@proception.ai, jayli@proception.ai, j.li@proception.ai, jayl@proception.ai</t>
+  </si>
+  <si>
     <t xml:space="preserve">Mbodi AI</t>
   </si>
   <si>
@@ -573,6 +732,15 @@
     <t xml:space="preserve">https://www.ycombinator.com/companies/mbodi-ai</t>
   </si>
   <si>
+    <t xml:space="preserve">mbodi.ai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://github.com/sebjperalta/mparse/commit/6fbd50331472a89c198b4bcf2df445c2bb668e79</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sebastian@mbodi.ai, sebastian.peralta@mbodi.ai, speralta@mbodi.ai, sebastianperalta@mbodi.ai, s.peralta@mbodi.ai, sebastianp@mbodi.ai</t>
+  </si>
+  <si>
     <t xml:space="preserve">Orangewood Labs</t>
   </si>
   <si>
@@ -606,6 +774,15 @@
     <t xml:space="preserve">https://www.ycombinator.com/companies/orangewood-labs</t>
   </si>
   <si>
+    <t xml:space="preserve">hellorobot@orangewood.co</t>
+  </si>
+  <si>
+    <t xml:space="preserve">orangewood.co</t>
+  </si>
+  <si>
+    <t xml:space="preserve">abhinav@orangewood.co, abhi@orangewood.co, abhinav.das@orangewood.co, adas@orangewood.co, abhinavdas@orangewood.co, a.das@orangewood.co</t>
+  </si>
+  <si>
     <t xml:space="preserve">Revise Robotics</t>
   </si>
   <si>
@@ -639,6 +816,12 @@
     <t xml:space="preserve">https://www.ycombinator.com/companies/revise-robotics</t>
   </si>
   <si>
+    <t xml:space="preserve">reviserobotics.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rupesh@reviserobotics.com, rupesh.jeyaram@reviserobotics.com, rjeyaram@reviserobotics.com, rupeshjeyaram@reviserobotics.com, r.jeyaram@reviserobotics.com, rupeshj@reviserobotics.com</t>
+  </si>
+  <si>
     <t xml:space="preserve">Aktoria Robotics</t>
   </si>
   <si>
@@ -672,6 +855,15 @@
     <t xml:space="preserve">https://www.ycombinator.com/companies/aktoria-robotics</t>
   </si>
   <si>
+    <t xml:space="preserve">aktoria.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://aktoria.com | personal guess: shreenabh@aktoria.com (prior {first} (11/11 indexed domains) (no personal addresses at this domain on site, DNS, YC, HN, Wayback, web or GitHub))</t>
+  </si>
+  <si>
+    <t xml:space="preserve">shreenabh@aktoria.com, shreenabh.agrawal@aktoria.com, sagrawal@aktoria.com, shreenabhagrawal@aktoria.com, s.agrawal@aktoria.com, shreenabha@aktoria.com</t>
+  </si>
+  <si>
     <t xml:space="preserve">Starcloud</t>
   </si>
   <si>
@@ -705,6 +897,15 @@
     <t xml:space="preserve">https://www.ycombinator.com/companies/starcloud</t>
   </si>
   <si>
+    <t xml:space="preserve">starcloud.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://github.com/adi-oltean/fastcad/commit/b49cf0f7c5adc950c21758fcec17c5c7c3fbaf4c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">adi@starcloud.com, adi.oltean@starcloud.com, aoltean@starcloud.com, adioltean@starcloud.com, a.oltean@starcloud.com, adio@starcloud.com</t>
+  </si>
+  <si>
     <t xml:space="preserve">Feather</t>
   </si>
   <si>
@@ -738,6 +939,15 @@
     <t xml:space="preserve">https://www.ycombinator.com/companies/feather</t>
   </si>
   <si>
+    <t xml:space="preserve">featherhq.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://github.com/aahan-feather/debt-collection/commit/15cfd1b5eb8e9aa6db5fa7a3c8c3328a53101d75</t>
+  </si>
+  <si>
+    <t xml:space="preserve">aahan@featherhq.com, aahan.sawhney@featherhq.com, asawhney@featherhq.com, aahansawhney@featherhq.com, a.sawhney@featherhq.com, aahans@featherhq.com</t>
+  </si>
+  <si>
     <t xml:space="preserve">Silurian</t>
   </si>
   <si>
@@ -774,6 +984,15 @@
     <t xml:space="preserve">https://www.ycombinator.com/companies/silurian</t>
   </si>
   <si>
+    <t xml:space="preserve">silurian.ai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pattern {first} from jayesh@silurian.ai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nikhil@silurian.ai, nikhil.shankar@silurian.ai, nshankar@silurian.ai, nikhilshankar@silurian.ai, n.shankar@silurian.ai, nikhils@silurian.ai</t>
+  </si>
+  <si>
     <t xml:space="preserve">Metric</t>
   </si>
   <si>
@@ -820,6 +1039,9 @@
   </si>
   <si>
     <t xml:space="preserve">Yellow columns on Tracker are yours to edit: Status, Date sent, Follow-up sent, Response, Notes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Email, Email status and the columns after Draft BCC belong to the email finder (finder.py). Draft To / Draft BCC are who the Gmail draft is actually addressed to.</t>
   </si>
   <si>
     <t xml:space="preserve">Claude regenerates everything else each batch and keeps what you typed in the yellow columns.</t>
@@ -1299,7 +1521,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:V21"/>
+  <dimension ref="A1:AC21"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
@@ -1322,9 +1544,16 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="0" width="30"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="0" width="26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="0" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="24" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="27" style="0" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="28" min="28" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="29" min="29" style="0" width="50"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1390,6 +1619,27 @@
       </c>
       <c r="V1" s="1" t="s">
         <v>21</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="AB1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="AC1" s="1" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1400,38 +1650,38 @@
         <v>1</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="K2" s="2"/>
       <c r="L2" s="2" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="N2" s="3" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="O2" s="4"/>
       <c r="P2" s="5" t="str">
@@ -1441,16 +1691,35 @@
       <c r="Q2" s="4"/>
       <c r="R2" s="3"/>
       <c r="S2" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="T2" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="U2" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="V2" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="W2" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="T2" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="U2" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="V2" s="6" t="s">
-        <v>36</v>
+      <c r="X2" s="2"/>
+      <c r="Y2" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="Z2" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="AA2" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="AB2" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="AC2" s="2" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1461,38 +1730,38 @@
         <v>1</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>38</v>
+        <v>49</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>40</v>
+        <v>51</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>41</v>
+        <v>52</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>42</v>
+        <v>53</v>
       </c>
       <c r="K3" s="2"/>
       <c r="L3" s="2" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="N3" s="3" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="O3" s="4"/>
       <c r="P3" s="5" t="str">
@@ -1502,16 +1771,35 @@
       <c r="Q3" s="4"/>
       <c r="R3" s="3"/>
       <c r="S3" s="3" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="T3" s="2" t="s">
-        <v>45</v>
+        <v>56</v>
       </c>
       <c r="U3" s="6" t="s">
-        <v>46</v>
+        <v>57</v>
       </c>
       <c r="V3" s="6" t="s">
-        <v>47</v>
+        <v>58</v>
+      </c>
+      <c r="W3" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="X3" s="2"/>
+      <c r="Y3" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="Z3" s="2" t="n">
+        <v>95</v>
+      </c>
+      <c r="AA3" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="AB3" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="AC3" s="2" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1522,40 +1810,40 @@
         <v>1</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>48</v>
+        <v>63</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>49</v>
+        <v>64</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="G4" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="H4" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="H4" s="2" t="s">
-        <v>40</v>
-      </c>
       <c r="I4" s="2" t="s">
-        <v>52</v>
+        <v>67</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>53</v>
+        <v>68</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>54</v>
+        <v>69</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="N4" s="3" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="O4" s="4"/>
       <c r="P4" s="5" t="str">
@@ -1565,16 +1853,35 @@
       <c r="Q4" s="4"/>
       <c r="R4" s="3"/>
       <c r="S4" s="3" t="s">
-        <v>56</v>
+        <v>71</v>
       </c>
       <c r="T4" s="2" t="s">
-        <v>57</v>
+        <v>72</v>
       </c>
       <c r="U4" s="6" t="s">
-        <v>58</v>
+        <v>73</v>
       </c>
       <c r="V4" s="6" t="s">
-        <v>59</v>
+        <v>74</v>
+      </c>
+      <c r="W4" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="X4" s="2"/>
+      <c r="Y4" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="Z4" s="2" t="n">
+        <v>95</v>
+      </c>
+      <c r="AA4" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="AB4" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="AC4" s="2" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1585,40 +1892,40 @@
         <v>1</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>60</v>
+        <v>78</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>49</v>
+        <v>64</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>62</v>
+        <v>80</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>63</v>
+        <v>81</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>64</v>
+        <v>82</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>65</v>
+        <v>83</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>67</v>
+        <v>85</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>68</v>
+        <v>86</v>
       </c>
       <c r="N5" s="3" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="O5" s="4"/>
       <c r="P5" s="5" t="str">
@@ -1628,16 +1935,37 @@
       <c r="Q5" s="4"/>
       <c r="R5" s="3"/>
       <c r="S5" s="3" t="s">
-        <v>69</v>
+        <v>87</v>
       </c>
       <c r="T5" s="2" t="s">
-        <v>70</v>
+        <v>88</v>
       </c>
       <c r="U5" s="6" t="s">
-        <v>71</v>
+        <v>89</v>
       </c>
       <c r="V5" s="6" t="s">
-        <v>72</v>
+        <v>90</v>
+      </c>
+      <c r="W5" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="X5" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="Y5" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="Z5" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="AA5" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="AB5" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="AC5" s="2" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1648,40 +1976,40 @@
         <v>1</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>73</v>
+        <v>95</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>49</v>
+        <v>64</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>74</v>
+        <v>96</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>75</v>
+        <v>97</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>76</v>
+        <v>98</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>77</v>
+        <v>99</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>78</v>
+        <v>100</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>79</v>
+        <v>101</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>80</v>
+        <v>102</v>
       </c>
       <c r="N6" s="3" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="O6" s="4"/>
       <c r="P6" s="5" t="str">
@@ -1691,19 +2019,40 @@
       <c r="Q6" s="4"/>
       <c r="R6" s="3"/>
       <c r="S6" s="3" t="s">
-        <v>81</v>
+        <v>103</v>
       </c>
       <c r="T6" s="2" t="s">
-        <v>82</v>
+        <v>104</v>
       </c>
       <c r="U6" s="6" t="s">
-        <v>83</v>
+        <v>105</v>
       </c>
       <c r="V6" s="6" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>106</v>
+      </c>
+      <c r="W6" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="X6" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="Y6" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="Z6" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="AA6" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="AB6" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="AC6" s="2" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="n">
         <v>6</v>
       </c>
@@ -1711,38 +2060,38 @@
         <v>1</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>85</v>
+        <v>111</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>86</v>
+        <v>112</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>87</v>
+        <v>113</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>88</v>
+        <v>114</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>89</v>
+        <v>115</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>90</v>
+        <v>116</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>91</v>
+        <v>117</v>
       </c>
       <c r="K7" s="2"/>
       <c r="L7" s="2" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>92</v>
+        <v>118</v>
       </c>
       <c r="N7" s="3" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="O7" s="4"/>
       <c r="P7" s="5" t="str">
@@ -1752,19 +2101,40 @@
       <c r="Q7" s="4"/>
       <c r="R7" s="3"/>
       <c r="S7" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="T7" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="U7" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="V7" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="W7" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="X7" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="Y7" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="Z7" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="AA7" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="T7" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="U7" s="6" t="s">
-        <v>95</v>
-      </c>
-      <c r="V7" s="6" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="AB7" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="AC7" s="2" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="n">
         <v>7</v>
       </c>
@@ -1772,38 +2142,38 @@
         <v>1</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>97</v>
+        <v>126</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>98</v>
+        <v>127</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>99</v>
+        <v>128</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>100</v>
+        <v>129</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>101</v>
+        <v>130</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>40</v>
+        <v>115</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>102</v>
+        <v>131</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>103</v>
+        <v>132</v>
       </c>
       <c r="K8" s="2"/>
       <c r="L8" s="2" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>104</v>
+        <v>133</v>
       </c>
       <c r="N8" s="3" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="O8" s="4"/>
       <c r="P8" s="5" t="str">
@@ -1813,19 +2183,40 @@
       <c r="Q8" s="4"/>
       <c r="R8" s="3"/>
       <c r="S8" s="3" t="s">
-        <v>105</v>
+        <v>134</v>
       </c>
       <c r="T8" s="2" t="s">
-        <v>106</v>
+        <v>135</v>
       </c>
       <c r="U8" s="6" t="s">
-        <v>107</v>
+        <v>136</v>
       </c>
       <c r="V8" s="6" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>137</v>
+      </c>
+      <c r="W8" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="X8" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="Y8" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="Z8" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="AA8" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="AB8" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="AC8" s="2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="n">
         <v>8</v>
       </c>
@@ -1833,38 +2224,38 @@
         <v>1</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>109</v>
+        <v>142</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>110</v>
+        <v>143</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>111</v>
+        <v>144</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>89</v>
+        <v>115</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>112</v>
+        <v>145</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>113</v>
+        <v>146</v>
       </c>
       <c r="K9" s="2"/>
       <c r="L9" s="2" t="s">
-        <v>114</v>
+        <v>147</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>115</v>
+        <v>148</v>
       </c>
       <c r="N9" s="3" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="O9" s="4"/>
       <c r="P9" s="5" t="str">
@@ -1874,16 +2265,35 @@
       <c r="Q9" s="4"/>
       <c r="R9" s="3"/>
       <c r="S9" s="3" t="s">
-        <v>116</v>
+        <v>149</v>
       </c>
       <c r="T9" s="2" t="s">
-        <v>117</v>
+        <v>150</v>
       </c>
       <c r="U9" s="6" t="s">
-        <v>118</v>
+        <v>151</v>
       </c>
       <c r="V9" s="6" t="s">
-        <v>119</v>
+        <v>152</v>
+      </c>
+      <c r="W9" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="X9" s="2"/>
+      <c r="Y9" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="Z9" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="AA9" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="AB9" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="AC9" s="2" t="s">
+        <v>156</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1894,38 +2304,38 @@
         <v>1</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>120</v>
+        <v>157</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>98</v>
+        <v>127</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>121</v>
+        <v>158</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>100</v>
+        <v>129</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>122</v>
+        <v>159</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>40</v>
+        <v>51</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>123</v>
+        <v>160</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>124</v>
+        <v>161</v>
       </c>
       <c r="K10" s="2"/>
       <c r="L10" s="2" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>125</v>
+        <v>162</v>
       </c>
       <c r="N10" s="3" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="O10" s="4"/>
       <c r="P10" s="5" t="str">
@@ -1935,19 +2345,38 @@
       <c r="Q10" s="4"/>
       <c r="R10" s="3"/>
       <c r="S10" s="3" t="s">
-        <v>126</v>
+        <v>163</v>
       </c>
       <c r="T10" s="2" t="s">
-        <v>127</v>
+        <v>164</v>
       </c>
       <c r="U10" s="6" t="s">
-        <v>128</v>
+        <v>165</v>
       </c>
       <c r="V10" s="6" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>166</v>
+      </c>
+      <c r="W10" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="X10" s="2"/>
+      <c r="Y10" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="Z10" s="2" t="n">
+        <v>95</v>
+      </c>
+      <c r="AA10" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="AB10" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="AC10" s="2" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="n">
         <v>10</v>
       </c>
@@ -1955,38 +2384,38 @@
         <v>1</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>130</v>
+        <v>171</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>98</v>
+        <v>127</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>131</v>
+        <v>172</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>62</v>
+        <v>80</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>132</v>
+        <v>173</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>133</v>
+        <v>51</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>134</v>
+        <v>174</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>135</v>
+        <v>175</v>
       </c>
       <c r="K11" s="2"/>
       <c r="L11" s="2" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>136</v>
+        <v>176</v>
       </c>
       <c r="N11" s="3" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="O11" s="4"/>
       <c r="P11" s="5" t="str">
@@ -1996,19 +2425,38 @@
       <c r="Q11" s="4"/>
       <c r="R11" s="3"/>
       <c r="S11" s="3" t="s">
-        <v>137</v>
+        <v>177</v>
       </c>
       <c r="T11" s="2" t="s">
-        <v>138</v>
+        <v>178</v>
       </c>
       <c r="U11" s="6" t="s">
-        <v>139</v>
+        <v>179</v>
       </c>
       <c r="V11" s="6" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>180</v>
+      </c>
+      <c r="W11" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="X11" s="2"/>
+      <c r="Y11" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="Z11" s="2" t="n">
+        <v>95</v>
+      </c>
+      <c r="AA11" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="AB11" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="AC11" s="2" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="n">
         <v>11</v>
       </c>
@@ -2016,38 +2464,38 @@
         <v>1</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>141</v>
+        <v>183</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>142</v>
+        <v>184</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>100</v>
+        <v>129</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>143</v>
+        <v>185</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>144</v>
+        <v>186</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>145</v>
+        <v>187</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>146</v>
+        <v>188</v>
       </c>
       <c r="K12" s="2"/>
       <c r="L12" s="2" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="M12" s="2" t="s">
-        <v>147</v>
+        <v>189</v>
       </c>
       <c r="N12" s="3" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="O12" s="4"/>
       <c r="P12" s="5" t="str">
@@ -2057,19 +2505,40 @@
       <c r="Q12" s="4"/>
       <c r="R12" s="3"/>
       <c r="S12" s="3" t="s">
-        <v>148</v>
+        <v>190</v>
       </c>
       <c r="T12" s="2" t="s">
-        <v>149</v>
+        <v>191</v>
       </c>
       <c r="U12" s="6" t="s">
-        <v>150</v>
+        <v>192</v>
       </c>
       <c r="V12" s="6" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>193</v>
+      </c>
+      <c r="W12" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="X12" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="Y12" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="Z12" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="AA12" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="AB12" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="AC12" s="2" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="n">
         <v>12</v>
       </c>
@@ -2077,38 +2546,38 @@
         <v>1</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>152</v>
+        <v>198</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>153</v>
+        <v>199</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>154</v>
+        <v>200</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>89</v>
+        <v>115</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>155</v>
+        <v>201</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>156</v>
+        <v>202</v>
       </c>
       <c r="K13" s="2"/>
       <c r="L13" s="2" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="M13" s="2" t="s">
-        <v>157</v>
+        <v>203</v>
       </c>
       <c r="N13" s="3" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="O13" s="4"/>
       <c r="P13" s="5" t="str">
@@ -2118,16 +2587,37 @@
       <c r="Q13" s="4"/>
       <c r="R13" s="3"/>
       <c r="S13" s="3" t="s">
-        <v>158</v>
+        <v>204</v>
       </c>
       <c r="T13" s="2" t="s">
-        <v>159</v>
+        <v>205</v>
       </c>
       <c r="U13" s="6" t="s">
-        <v>160</v>
+        <v>206</v>
       </c>
       <c r="V13" s="6" t="s">
-        <v>161</v>
+        <v>207</v>
+      </c>
+      <c r="W13" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="X13" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="Y13" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="Z13" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="AA13" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="AB13" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="AC13" s="2" t="s">
+        <v>211</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2138,38 +2628,38 @@
         <v>1</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>162</v>
+        <v>212</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>98</v>
+        <v>127</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>163</v>
+        <v>213</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>100</v>
+        <v>129</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>164</v>
+        <v>214</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>40</v>
+        <v>51</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>165</v>
+        <v>215</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>166</v>
+        <v>216</v>
       </c>
       <c r="K14" s="2"/>
       <c r="L14" s="2" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="M14" s="2" t="s">
-        <v>167</v>
+        <v>217</v>
       </c>
       <c r="N14" s="3" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="O14" s="4"/>
       <c r="P14" s="5" t="str">
@@ -2179,16 +2669,35 @@
       <c r="Q14" s="4"/>
       <c r="R14" s="3"/>
       <c r="S14" s="3" t="s">
-        <v>168</v>
+        <v>218</v>
       </c>
       <c r="T14" s="2" t="s">
-        <v>169</v>
+        <v>219</v>
       </c>
       <c r="U14" s="6" t="s">
-        <v>170</v>
+        <v>220</v>
       </c>
       <c r="V14" s="6" t="s">
-        <v>171</v>
+        <v>221</v>
+      </c>
+      <c r="W14" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="X14" s="2"/>
+      <c r="Y14" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="Z14" s="2" t="n">
+        <v>95</v>
+      </c>
+      <c r="AA14" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="AB14" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="AC14" s="2" t="s">
+        <v>224</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2199,38 +2708,38 @@
         <v>1</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>172</v>
+        <v>225</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>173</v>
+        <v>226</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>100</v>
+        <v>129</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>174</v>
+        <v>227</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>40</v>
+        <v>51</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>175</v>
+        <v>228</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>176</v>
+        <v>229</v>
       </c>
       <c r="K15" s="2"/>
       <c r="L15" s="2" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="M15" s="2" t="s">
-        <v>177</v>
+        <v>230</v>
       </c>
       <c r="N15" s="3" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="O15" s="4"/>
       <c r="P15" s="5" t="str">
@@ -2240,16 +2749,35 @@
       <c r="Q15" s="4"/>
       <c r="R15" s="3"/>
       <c r="S15" s="3" t="s">
-        <v>178</v>
+        <v>231</v>
       </c>
       <c r="T15" s="2" t="s">
-        <v>179</v>
+        <v>232</v>
       </c>
       <c r="U15" s="6" t="s">
-        <v>180</v>
+        <v>233</v>
       </c>
       <c r="V15" s="6" t="s">
-        <v>181</v>
+        <v>234</v>
+      </c>
+      <c r="W15" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="X15" s="2"/>
+      <c r="Y15" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="Z15" s="2" t="n">
+        <v>95</v>
+      </c>
+      <c r="AA15" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="AB15" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="AC15" s="2" t="s">
+        <v>237</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2260,38 +2788,38 @@
         <v>1</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>182</v>
+        <v>238</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>98</v>
+        <v>127</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>183</v>
+        <v>239</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>87</v>
+        <v>113</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>184</v>
+        <v>240</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>185</v>
+        <v>241</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>186</v>
+        <v>242</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>187</v>
+        <v>243</v>
       </c>
       <c r="K16" s="2"/>
       <c r="L16" s="2" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="M16" s="2" t="s">
-        <v>188</v>
+        <v>244</v>
       </c>
       <c r="N16" s="3" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="O16" s="4"/>
       <c r="P16" s="5" t="str">
@@ -2301,16 +2829,37 @@
       <c r="Q16" s="4"/>
       <c r="R16" s="3"/>
       <c r="S16" s="3" t="s">
-        <v>189</v>
+        <v>245</v>
       </c>
       <c r="T16" s="2" t="s">
-        <v>190</v>
+        <v>246</v>
       </c>
       <c r="U16" s="6" t="s">
-        <v>191</v>
+        <v>247</v>
       </c>
       <c r="V16" s="6" t="s">
-        <v>192</v>
+        <v>248</v>
+      </c>
+      <c r="W16" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="X16" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="Y16" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="Z16" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="AA16" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="AB16" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="AC16" s="2" t="s">
+        <v>251</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2321,40 +2870,40 @@
         <v>1</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>193</v>
+        <v>252</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>49</v>
+        <v>64</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>194</v>
+        <v>253</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>100</v>
+        <v>129</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>195</v>
+        <v>254</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>89</v>
+        <v>51</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>196</v>
+        <v>255</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>197</v>
+        <v>256</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>198</v>
+        <v>257</v>
       </c>
       <c r="L17" s="2" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="M17" s="2" t="s">
-        <v>199</v>
+        <v>258</v>
       </c>
       <c r="N17" s="3" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="O17" s="4"/>
       <c r="P17" s="5" t="str">
@@ -2364,19 +2913,38 @@
       <c r="Q17" s="4"/>
       <c r="R17" s="3"/>
       <c r="S17" s="3" t="s">
-        <v>200</v>
+        <v>259</v>
       </c>
       <c r="T17" s="2" t="s">
-        <v>201</v>
+        <v>260</v>
       </c>
       <c r="U17" s="6" t="s">
-        <v>202</v>
+        <v>261</v>
       </c>
       <c r="V17" s="6" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>262</v>
+      </c>
+      <c r="W17" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="X17" s="2"/>
+      <c r="Y17" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="Z17" s="2" t="n">
+        <v>96</v>
+      </c>
+      <c r="AA17" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="AB17" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="AC17" s="2" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="n">
         <v>17</v>
       </c>
@@ -2384,38 +2952,38 @@
         <v>1</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>204</v>
+        <v>265</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>205</v>
+        <v>266</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>87</v>
+        <v>113</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>206</v>
+        <v>267</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>207</v>
+        <v>268</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>208</v>
+        <v>269</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>209</v>
+        <v>270</v>
       </c>
       <c r="K18" s="2"/>
       <c r="L18" s="2" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="M18" s="2" t="s">
-        <v>210</v>
+        <v>271</v>
       </c>
       <c r="N18" s="3" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="O18" s="4"/>
       <c r="P18" s="5" t="str">
@@ -2425,16 +2993,35 @@
       <c r="Q18" s="4"/>
       <c r="R18" s="3"/>
       <c r="S18" s="3" t="s">
-        <v>211</v>
+        <v>272</v>
       </c>
       <c r="T18" s="2" t="s">
-        <v>212</v>
+        <v>273</v>
       </c>
       <c r="U18" s="6" t="s">
-        <v>213</v>
+        <v>274</v>
       </c>
       <c r="V18" s="6" t="s">
-        <v>214</v>
+        <v>275</v>
+      </c>
+      <c r="W18" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="X18" s="2"/>
+      <c r="Y18" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="Z18" s="2" t="n">
+        <v>99</v>
+      </c>
+      <c r="AA18" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="AB18" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="AC18" s="2" t="s">
+        <v>278</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2445,38 +3032,38 @@
         <v>1</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>215</v>
+        <v>279</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>216</v>
+        <v>280</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>217</v>
+        <v>281</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>218</v>
+        <v>282</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>40</v>
+        <v>51</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>219</v>
+        <v>283</v>
       </c>
       <c r="J19" s="2" t="s">
-        <v>220</v>
+        <v>284</v>
       </c>
       <c r="K19" s="2"/>
       <c r="L19" s="2" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="M19" s="2" t="s">
-        <v>221</v>
+        <v>285</v>
       </c>
       <c r="N19" s="3" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="O19" s="4"/>
       <c r="P19" s="5" t="str">
@@ -2486,16 +3073,35 @@
       <c r="Q19" s="4"/>
       <c r="R19" s="3"/>
       <c r="S19" s="3" t="s">
-        <v>222</v>
+        <v>286</v>
       </c>
       <c r="T19" s="2" t="s">
-        <v>223</v>
+        <v>287</v>
       </c>
       <c r="U19" s="6" t="s">
-        <v>224</v>
+        <v>288</v>
       </c>
       <c r="V19" s="6" t="s">
-        <v>225</v>
+        <v>289</v>
+      </c>
+      <c r="W19" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="X19" s="2"/>
+      <c r="Y19" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="Z19" s="2" t="n">
+        <v>95</v>
+      </c>
+      <c r="AA19" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="AB19" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="AC19" s="2" t="s">
+        <v>292</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2506,38 +3112,38 @@
         <v>1</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>226</v>
+        <v>293</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>98</v>
+        <v>127</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>227</v>
+        <v>294</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>228</v>
+        <v>295</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>229</v>
+        <v>296</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>40</v>
+        <v>51</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>230</v>
+        <v>297</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>231</v>
+        <v>298</v>
       </c>
       <c r="K20" s="2"/>
       <c r="L20" s="2" t="s">
-        <v>114</v>
+        <v>147</v>
       </c>
       <c r="M20" s="2" t="s">
-        <v>232</v>
+        <v>299</v>
       </c>
       <c r="N20" s="3" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="O20" s="4"/>
       <c r="P20" s="5" t="str">
@@ -2547,16 +3153,35 @@
       <c r="Q20" s="4"/>
       <c r="R20" s="3"/>
       <c r="S20" s="3" t="s">
-        <v>233</v>
+        <v>300</v>
       </c>
       <c r="T20" s="2" t="s">
-        <v>234</v>
+        <v>301</v>
       </c>
       <c r="U20" s="6" t="s">
-        <v>235</v>
+        <v>302</v>
       </c>
       <c r="V20" s="6" t="s">
-        <v>236</v>
+        <v>303</v>
+      </c>
+      <c r="W20" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="X20" s="2"/>
+      <c r="Y20" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="Z20" s="2" t="n">
+        <v>95</v>
+      </c>
+      <c r="AA20" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="AB20" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="AC20" s="2" t="s">
+        <v>306</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2567,38 +3192,38 @@
         <v>1</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>237</v>
+        <v>307</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>98</v>
+        <v>127</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>238</v>
+        <v>308</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>239</v>
+        <v>309</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>240</v>
+        <v>310</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>40</v>
+        <v>115</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>241</v>
+        <v>311</v>
       </c>
       <c r="J21" s="2" t="s">
-        <v>242</v>
+        <v>312</v>
       </c>
       <c r="K21" s="2"/>
       <c r="L21" s="2" t="s">
-        <v>243</v>
+        <v>313</v>
       </c>
       <c r="M21" s="2" t="s">
-        <v>244</v>
+        <v>314</v>
       </c>
       <c r="N21" s="3" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="O21" s="4"/>
       <c r="P21" s="5" t="str">
@@ -2608,20 +3233,39 @@
       <c r="Q21" s="4"/>
       <c r="R21" s="3"/>
       <c r="S21" s="3" t="s">
-        <v>245</v>
+        <v>315</v>
       </c>
       <c r="T21" s="2" t="s">
-        <v>246</v>
+        <v>316</v>
       </c>
       <c r="U21" s="6" t="s">
-        <v>247</v>
+        <v>317</v>
       </c>
       <c r="V21" s="6" t="s">
-        <v>248</v>
+        <v>318</v>
+      </c>
+      <c r="W21" s="2" t="s">
+        <v>310</v>
+      </c>
+      <c r="X21" s="2"/>
+      <c r="Y21" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="Z21" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="AA21" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="AB21" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="AC21" s="2" t="s">
+        <v>321</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:V21"/>
+  <autoFilter ref="A1:AC21"/>
   <dataValidations count="1">
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="N2:N21" type="list">
       <formula1>"Waiting on build,Ready to review,Verified,Sent,Followed up,Replied,Call scheduled,No reply,Skip"</formula1>
@@ -2695,15 +3339,15 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>249</v>
+        <v>322</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>250</v>
+        <v>323</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>251</v>
+        <v>324</v>
       </c>
       <c r="B2" s="8" t="n">
         <f aca="false">COUNTA(Tracker!C2:C21)</f>
@@ -2712,7 +3356,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>252</v>
+        <v>325</v>
       </c>
       <c r="B3" s="8" t="n">
         <f aca="false">COUNTIF(Tracker!N2:N21,"Waiting on build")</f>
@@ -2721,7 +3365,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="B4" s="8" t="n">
         <f aca="false">COUNTIF(Tracker!N2:N21,"Ready to review")</f>
@@ -2730,7 +3374,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>253</v>
+        <v>326</v>
       </c>
       <c r="B5" s="8" t="n">
         <f aca="false">COUNTIF(Tracker!N2:N21,"Verified")</f>
@@ -2739,7 +3383,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>254</v>
+        <v>327</v>
       </c>
       <c r="B6" s="8" t="n">
         <f aca="false">COUNTIF(Tracker!N2:N21,"Sent")</f>
@@ -2748,7 +3392,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>255</v>
+        <v>328</v>
       </c>
       <c r="B7" s="8" t="n">
         <f aca="false">COUNTIF(Tracker!N2:N21,"Followed up")</f>
@@ -2757,7 +3401,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>256</v>
+        <v>329</v>
       </c>
       <c r="B8" s="8" t="n">
         <f aca="false">COUNTIF(Tracker!N2:N21,"Replied")</f>
@@ -2766,7 +3410,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>257</v>
+        <v>330</v>
       </c>
       <c r="B9" s="8" t="n">
         <f aca="false">COUNTIF(Tracker!N2:N21,"Call scheduled")</f>
@@ -2775,7 +3419,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>258</v>
+        <v>331</v>
       </c>
       <c r="B10" s="8" t="n">
         <f aca="false">COUNTIF(Tracker!N2:N21,"No reply")</f>
@@ -2784,7 +3428,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>259</v>
+        <v>332</v>
       </c>
       <c r="B11" s="8" t="n">
         <f aca="false">COUNTIF(Tracker!N2:N21,"Skip")</f>
@@ -2797,7 +3441,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>260</v>
+        <v>333</v>
       </c>
       <c r="B13" s="8" t="n">
         <f aca="false">COUNTIF(Tracker!D2:D21,"A")</f>
@@ -2806,7 +3450,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="8" t="s">
-        <v>261</v>
+        <v>334</v>
       </c>
       <c r="B14" s="8" t="n">
         <f aca="false">COUNTIF(Tracker!D2:D21,"B")</f>
@@ -2815,7 +3459,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="s">
-        <v>262</v>
+        <v>335</v>
       </c>
       <c r="B15" s="8" t="n">
         <f aca="false">COUNTIF(Tracker!D2:D21,"C")</f>
@@ -2828,7 +3472,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="s">
-        <v>263</v>
+        <v>336</v>
       </c>
       <c r="B17" s="9" t="str">
         <f aca="false">IFERROR((B8+B9)/(B6+B7+B8+B9+B10),"-")</f>
@@ -2851,7 +3495,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="110"/>
@@ -2859,42 +3503,47 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
-        <v>264</v>
+        <v>337</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>265</v>
+        <v>338</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>266</v>
+        <v>339</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>267</v>
+        <v>340</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>268</v>
+        <v>341</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>269</v>
+        <v>342</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>270</v>
+        <v>343</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>271</v>
+        <v>344</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="8" t="s">
+        <v>345</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Batch 2: verify site claims, fix 5 openers, 9 Gmail drafts created
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K6KjNKe9qCXHsofcBCunE2
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -1080,10 +1080,10 @@
     <t xml:space="preserve">Camera-driven robot finishing (grinding, cutting, sanding) and inspection for foundries and aerospace. 10+ robots at a cast-iron foundry.</t>
   </si>
   <si>
-    <t xml:space="preserve">Homepage stats '100x Faster' and '&lt;2 Year ROI' have no baseline or example; one sentence each would make them believable.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The '100x faster' stat on pivotrobotics.com</t>
+    <t xml:space="preserve">'100x Faster' stat refers to adding a new part without programming (small caption), but the big number reads like grinding speed (verified).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Your '100x Faster' stat might get misread</t>
   </si>
   <si>
     <t xml:space="preserve">SWE roles need 1+ yr.</t>
@@ -1140,10 +1140,10 @@
     <t xml:space="preserve">Voxel Series-1, a home robot that tidies. Founder ex-Boston Dynamics Spot manipulation.</t>
   </si>
   <si>
-    <t xml:space="preserve">Homepage has both 'Shop' and 'Reserve' with no price, availability date, or what reserving means.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">'Shop' vs 'Reserve' for Voxel</t>
+    <t xml:space="preserve">Homepage has 'Shop' and 'How Do I Get a Robot?' (goes to reserve) but no price, deposit, or availability date (verified).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How do I get a Voxel?</t>
   </si>
   <si>
     <t xml:space="preserve">Only an open call in NYC.</t>
@@ -1260,7 +1260,7 @@
     <t xml:space="preserve">Sells and leases robots and parts with fast delivery, plus teleop data collection, RL environments and an eval stack.</t>
   </si>
   <si>
-    <t xml:space="preserve">roboticscenter.ai gives three different platform counts (30+, 60+, 90+) and its headline promises 48-hour delivery while the YC page says 72. Robotics Engineer Intern posting.</t>
+    <t xml:space="preserve">roboticscenter.ai body text gives three platform counts (30+ stats bar, 60+ how-it-works, 90+ store card; verified) and its headline promises 48-hour delivery while the YC page says 72. Robotics Engineer Intern posting.</t>
   </si>
   <si>
     <t xml:space="preserve">Aug 15 thread (jerry@deepawareai.com). Robotics Engineer Intern.</t>
@@ -1419,7 +1419,7 @@
     <t xml:space="preserve">AI systems-engineering (SysML v2 MBSE) software: requirements, architecture, analysis, V&amp;V, safety. Free Pro plan for students.</t>
   </si>
   <si>
-    <t xml:space="preserve">Free Pro plan for students. Offer: model the VEX robot in Dalus and send a write-up of where a student gets stuck. Pricing page 'Try for free' buttons lead to the demo form.</t>
+    <t xml:space="preserve">Free Pro plan for students needs a .edu email (Venkat is in high school, so the email asks). Offer: model the VEX robot in Dalus and send a write-up of where a student gets stuck. Pricing page 'Try for free' buttons lead to the demo form.</t>
   </si>
   <si>
     <t xml:space="preserve">Aug 15 thread. GTM Intern any level.</t>
@@ -1476,7 +1476,7 @@
     <t xml:space="preserve">AI agents that turn specs and drawings into electrical/control designs (single-lines, P&amp;IDs, BOMs), export DWG/DEXPI/JSON. Daikin customer.</t>
   </si>
   <si>
-    <t xml:space="preserve">Homepage examples tag the same pump P-1, P-101 and MP-1, which a controls engineer would notice on a page selling tag tracing.</t>
+    <t xml:space="preserve">No site issue used (checked: P-1/MP-1 is pump vs motor tag, P-101 is the sheet, so not an error). Hook: MTS Computer Vision / Graphics role open to any experience; Towaki's NVIDIA neural-fields background.</t>
   </si>
   <si>
     <t xml:space="preserve">Aug 15 thread. MTS CV/Graphics open to any level.</t>
@@ -1533,10 +1533,10 @@
     <t xml:space="preserve">Portable 'Sunrise' factories where robots assemble solar array bays on site (0.5-1 MW per shift).</t>
   </si>
   <si>
-    <t xml:space="preserve">Homepage responsibility list (Charge vs EPC) doesn't say who handles pile driving, which an EPC would ask first. Mechanical Engineer role open to new grads.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Who drives the piles?</t>
+    <t xml:space="preserve">Homepage responsibility list has three unlabeled columns, so readers infer that pile driving stays with the EPC (verified). Mechanical Engineer role open to new grads.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Charge vs. EPC columns on your homepage</t>
   </si>
   <si>
     <t xml:space="preserve">Bigger team (25), full-time roles.</t>
@@ -4445,7 +4445,7 @@
       </c>
       <c r="X29" s="2"/>
     </row>
-    <row r="30" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="n">
         <v>29</v>
       </c>
@@ -4774,7 +4774,7 @@
       </c>
       <c r="X34" s="2"/>
     </row>
-    <row r="35" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="n">
         <v>34</v>
       </c>
@@ -4900,7 +4900,7 @@
       </c>
       <c r="X36" s="2"/>
     </row>
-    <row r="37" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="2" t="n">
         <v>36</v>
       </c>

</xml_diff>